<commit_message>
iCoA register: pre-SOP certificates issued together on 13.05.2026
Head of QC, 05.09.2026: every certificate whose lot was packed before the
SOP floor is issued on one day, 13.05.2026 (a Wednesday), in chronological
order of packaging — iCoA-PP_26-001 to -118 — and the lots packed after it
follow on their last day of packaging, -119 onward. The day comes from
--batch-issue= (weekend refused). Lots the tracker leaves without a P
number take the list's P number so the sheet's date lookups find them.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/deliverables/qc_gap_analysis/tracker/iCoA_Issuance_Register_prelim.xlsx
+++ b/deliverables/qc_gap_analysis/tracker/iCoA_Issuance_Register_prelim.xlsx
@@ -689,7 +689,7 @@
         <v/>
       </c>
       <c r="E2" s="5">
-        <f>IF(AND(C2="yes",ISNUMBER(G2)),MAX(DATE(2026,5,11),G2),"")</f>
+        <f>IF(AND(C2="yes",ISNUMBER(G2)),MAX(DATE(2026,5,13),G2),"")</f>
         <v/>
       </c>
       <c r="F2" s="5">
@@ -780,7 +780,7 @@
         <v/>
       </c>
       <c r="E3" s="5">
-        <f>IF(AND(C3="yes",ISNUMBER(G3)),MAX(DATE(2026,5,11),G3),"")</f>
+        <f>IF(AND(C3="yes",ISNUMBER(G3)),MAX(DATE(2026,5,13),G3),"")</f>
         <v/>
       </c>
       <c r="F3" s="5">
@@ -871,7 +871,7 @@
         <v/>
       </c>
       <c r="E4" s="5">
-        <f>IF(AND(C4="yes",ISNUMBER(G4)),MAX(DATE(2026,5,11),G4),"")</f>
+        <f>IF(AND(C4="yes",ISNUMBER(G4)),MAX(DATE(2026,5,13),G4),"")</f>
         <v/>
       </c>
       <c r="F4" s="5">
@@ -962,7 +962,7 @@
         <v/>
       </c>
       <c r="E5" s="5">
-        <f>IF(AND(C5="yes",ISNUMBER(G5)),MAX(DATE(2026,5,11),G5),"")</f>
+        <f>IF(AND(C5="yes",ISNUMBER(G5)),MAX(DATE(2026,5,13),G5),"")</f>
         <v/>
       </c>
       <c r="F5" s="5">
@@ -1053,7 +1053,7 @@
         <v/>
       </c>
       <c r="E6" s="5">
-        <f>IF(AND(C6="yes",ISNUMBER(G6)),MAX(DATE(2026,5,11),G6),"")</f>
+        <f>IF(AND(C6="yes",ISNUMBER(G6)),MAX(DATE(2026,5,13),G6),"")</f>
         <v/>
       </c>
       <c r="F6" s="5">
@@ -1144,7 +1144,7 @@
         <v/>
       </c>
       <c r="E7" s="5">
-        <f>IF(AND(C7="yes",ISNUMBER(G7)),MAX(DATE(2026,5,11),G7),"")</f>
+        <f>IF(AND(C7="yes",ISNUMBER(G7)),MAX(DATE(2026,5,13),G7),"")</f>
         <v/>
       </c>
       <c r="F7" s="5">
@@ -1235,7 +1235,7 @@
         <v/>
       </c>
       <c r="E8" s="5">
-        <f>IF(AND(C8="yes",ISNUMBER(G8)),MAX(DATE(2026,5,11),G8),"")</f>
+        <f>IF(AND(C8="yes",ISNUMBER(G8)),MAX(DATE(2026,5,13),G8),"")</f>
         <v/>
       </c>
       <c r="F8" s="5">
@@ -1326,7 +1326,7 @@
         <v/>
       </c>
       <c r="E9" s="5">
-        <f>IF(AND(C9="yes",ISNUMBER(G9)),MAX(DATE(2026,5,11),G9),"")</f>
+        <f>IF(AND(C9="yes",ISNUMBER(G9)),MAX(DATE(2026,5,13),G9),"")</f>
         <v/>
       </c>
       <c r="F9" s="5">
@@ -1417,7 +1417,7 @@
         <v/>
       </c>
       <c r="E10" s="5">
-        <f>IF(AND(C10="yes",ISNUMBER(G10)),MAX(DATE(2026,5,11),G10),"")</f>
+        <f>IF(AND(C10="yes",ISNUMBER(G10)),MAX(DATE(2026,5,13),G10),"")</f>
         <v/>
       </c>
       <c r="F10" s="5">
@@ -1508,7 +1508,7 @@
         <v/>
       </c>
       <c r="E11" s="5">
-        <f>IF(AND(C11="yes",ISNUMBER(G11)),MAX(DATE(2026,5,11),G11),"")</f>
+        <f>IF(AND(C11="yes",ISNUMBER(G11)),MAX(DATE(2026,5,13),G11),"")</f>
         <v/>
       </c>
       <c r="F11" s="5">
@@ -1599,7 +1599,7 @@
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>IF(AND(C12="yes",ISNUMBER(G12)),MAX(DATE(2026,5,11),G12),"")</f>
+        <f>IF(AND(C12="yes",ISNUMBER(G12)),MAX(DATE(2026,5,13),G12),"")</f>
         <v/>
       </c>
       <c r="F12" s="5">
@@ -1690,7 +1690,7 @@
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>IF(AND(C13="yes",ISNUMBER(G13)),MAX(DATE(2026,5,11),G13),"")</f>
+        <f>IF(AND(C13="yes",ISNUMBER(G13)),MAX(DATE(2026,5,13),G13),"")</f>
         <v/>
       </c>
       <c r="F13" s="5">
@@ -1781,7 +1781,7 @@
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>IF(AND(C14="yes",ISNUMBER(G14)),MAX(DATE(2026,5,11),G14),"")</f>
+        <f>IF(AND(C14="yes",ISNUMBER(G14)),MAX(DATE(2026,5,13),G14),"")</f>
         <v/>
       </c>
       <c r="F14" s="5">
@@ -1872,7 +1872,7 @@
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>IF(AND(C15="yes",ISNUMBER(G15)),MAX(DATE(2026,5,11),G15),"")</f>
+        <f>IF(AND(C15="yes",ISNUMBER(G15)),MAX(DATE(2026,5,13),G15),"")</f>
         <v/>
       </c>
       <c r="F15" s="5">
@@ -1963,7 +1963,7 @@
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>IF(AND(C16="yes",ISNUMBER(G16)),MAX(DATE(2026,5,11),G16),"")</f>
+        <f>IF(AND(C16="yes",ISNUMBER(G16)),MAX(DATE(2026,5,13),G16),"")</f>
         <v/>
       </c>
       <c r="F16" s="5">
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>IF(AND(C17="yes",ISNUMBER(G17)),MAX(DATE(2026,5,11),G17),"")</f>
+        <f>IF(AND(C17="yes",ISNUMBER(G17)),MAX(DATE(2026,5,13),G17),"")</f>
         <v/>
       </c>
       <c r="F17" s="5">
@@ -2145,7 +2145,7 @@
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>IF(AND(C18="yes",ISNUMBER(G18)),MAX(DATE(2026,5,11),G18),"")</f>
+        <f>IF(AND(C18="yes",ISNUMBER(G18)),MAX(DATE(2026,5,13),G18),"")</f>
         <v/>
       </c>
       <c r="F18" s="5">
@@ -2236,7 +2236,7 @@
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>IF(AND(C19="yes",ISNUMBER(G19)),MAX(DATE(2026,5,11),G19),"")</f>
+        <f>IF(AND(C19="yes",ISNUMBER(G19)),MAX(DATE(2026,5,13),G19),"")</f>
         <v/>
       </c>
       <c r="F19" s="5">
@@ -2327,7 +2327,7 @@
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>IF(AND(C20="yes",ISNUMBER(G20)),MAX(DATE(2026,5,11),G20),"")</f>
+        <f>IF(AND(C20="yes",ISNUMBER(G20)),MAX(DATE(2026,5,13),G20),"")</f>
         <v/>
       </c>
       <c r="F20" s="5">
@@ -2418,7 +2418,7 @@
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>IF(AND(C21="yes",ISNUMBER(G21)),MAX(DATE(2026,5,11),G21),"")</f>
+        <f>IF(AND(C21="yes",ISNUMBER(G21)),MAX(DATE(2026,5,13),G21),"")</f>
         <v/>
       </c>
       <c r="F21" s="5">
@@ -2509,7 +2509,7 @@
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>IF(AND(C22="yes",ISNUMBER(G22)),MAX(DATE(2026,5,11),G22),"")</f>
+        <f>IF(AND(C22="yes",ISNUMBER(G22)),MAX(DATE(2026,5,13),G22),"")</f>
         <v/>
       </c>
       <c r="F22" s="5">
@@ -2600,7 +2600,7 @@
         <v/>
       </c>
       <c r="E23" s="5">
-        <f>IF(AND(C23="yes",ISNUMBER(G23)),MAX(DATE(2026,5,11),G23),"")</f>
+        <f>IF(AND(C23="yes",ISNUMBER(G23)),MAX(DATE(2026,5,13),G23),"")</f>
         <v/>
       </c>
       <c r="F23" s="5">
@@ -2691,7 +2691,7 @@
         <v/>
       </c>
       <c r="E24" s="5">
-        <f>IF(AND(C24="yes",ISNUMBER(G24)),MAX(DATE(2026,5,11),G24),"")</f>
+        <f>IF(AND(C24="yes",ISNUMBER(G24)),MAX(DATE(2026,5,13),G24),"")</f>
         <v/>
       </c>
       <c r="F24" s="5">
@@ -2782,7 +2782,7 @@
         <v/>
       </c>
       <c r="E25" s="5">
-        <f>IF(AND(C25="yes",ISNUMBER(G25)),MAX(DATE(2026,5,11),G25),"")</f>
+        <f>IF(AND(C25="yes",ISNUMBER(G25)),MAX(DATE(2026,5,13),G25),"")</f>
         <v/>
       </c>
       <c r="F25" s="5">
@@ -2873,7 +2873,7 @@
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>IF(AND(C26="yes",ISNUMBER(G26)),MAX(DATE(2026,5,11),G26),"")</f>
+        <f>IF(AND(C26="yes",ISNUMBER(G26)),MAX(DATE(2026,5,13),G26),"")</f>
         <v/>
       </c>
       <c r="F26" s="5">
@@ -2964,7 +2964,7 @@
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>IF(AND(C27="yes",ISNUMBER(G27)),MAX(DATE(2026,5,11),G27),"")</f>
+        <f>IF(AND(C27="yes",ISNUMBER(G27)),MAX(DATE(2026,5,13),G27),"")</f>
         <v/>
       </c>
       <c r="F27" s="5">
@@ -3055,7 +3055,7 @@
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>IF(AND(C28="yes",ISNUMBER(G28)),MAX(DATE(2026,5,11),G28),"")</f>
+        <f>IF(AND(C28="yes",ISNUMBER(G28)),MAX(DATE(2026,5,13),G28),"")</f>
         <v/>
       </c>
       <c r="F28" s="5">
@@ -3146,7 +3146,7 @@
         <v/>
       </c>
       <c r="E29" s="5">
-        <f>IF(AND(C29="yes",ISNUMBER(G29)),MAX(DATE(2026,5,11),G29),"")</f>
+        <f>IF(AND(C29="yes",ISNUMBER(G29)),MAX(DATE(2026,5,13),G29),"")</f>
         <v/>
       </c>
       <c r="F29" s="5">
@@ -3237,7 +3237,7 @@
         <v/>
       </c>
       <c r="E30" s="5">
-        <f>IF(AND(C30="yes",ISNUMBER(G30)),MAX(DATE(2026,5,11),G30),"")</f>
+        <f>IF(AND(C30="yes",ISNUMBER(G30)),MAX(DATE(2026,5,13),G30),"")</f>
         <v/>
       </c>
       <c r="F30" s="5">
@@ -3328,7 +3328,7 @@
         <v/>
       </c>
       <c r="E31" s="5">
-        <f>IF(AND(C31="yes",ISNUMBER(G31)),MAX(DATE(2026,5,11),G31),"")</f>
+        <f>IF(AND(C31="yes",ISNUMBER(G31)),MAX(DATE(2026,5,13),G31),"")</f>
         <v/>
       </c>
       <c r="F31" s="5">
@@ -3419,7 +3419,7 @@
         <v/>
       </c>
       <c r="E32" s="5">
-        <f>IF(AND(C32="yes",ISNUMBER(G32)),MAX(DATE(2026,5,11),G32),"")</f>
+        <f>IF(AND(C32="yes",ISNUMBER(G32)),MAX(DATE(2026,5,13),G32),"")</f>
         <v/>
       </c>
       <c r="F32" s="5">
@@ -3510,7 +3510,7 @@
         <v/>
       </c>
       <c r="E33" s="5">
-        <f>IF(AND(C33="yes",ISNUMBER(G33)),MAX(DATE(2026,5,11),G33),"")</f>
+        <f>IF(AND(C33="yes",ISNUMBER(G33)),MAX(DATE(2026,5,13),G33),"")</f>
         <v/>
       </c>
       <c r="F33" s="5">
@@ -3601,7 +3601,7 @@
         <v/>
       </c>
       <c r="E34" s="5">
-        <f>IF(AND(C34="yes",ISNUMBER(G34)),MAX(DATE(2026,5,11),G34),"")</f>
+        <f>IF(AND(C34="yes",ISNUMBER(G34)),MAX(DATE(2026,5,13),G34),"")</f>
         <v/>
       </c>
       <c r="F34" s="5">
@@ -3692,7 +3692,7 @@
         <v/>
       </c>
       <c r="E35" s="5">
-        <f>IF(AND(C35="yes",ISNUMBER(G35)),MAX(DATE(2026,5,11),G35),"")</f>
+        <f>IF(AND(C35="yes",ISNUMBER(G35)),MAX(DATE(2026,5,13),G35),"")</f>
         <v/>
       </c>
       <c r="F35" s="5">
@@ -3783,7 +3783,7 @@
         <v/>
       </c>
       <c r="E36" s="5">
-        <f>IF(AND(C36="yes",ISNUMBER(G36)),MAX(DATE(2026,5,11),G36),"")</f>
+        <f>IF(AND(C36="yes",ISNUMBER(G36)),MAX(DATE(2026,5,13),G36),"")</f>
         <v/>
       </c>
       <c r="F36" s="5">
@@ -3874,7 +3874,7 @@
         <v/>
       </c>
       <c r="E37" s="5">
-        <f>IF(AND(C37="yes",ISNUMBER(G37)),MAX(DATE(2026,5,11),G37),"")</f>
+        <f>IF(AND(C37="yes",ISNUMBER(G37)),MAX(DATE(2026,5,13),G37),"")</f>
         <v/>
       </c>
       <c r="F37" s="5">
@@ -3965,7 +3965,7 @@
         <v/>
       </c>
       <c r="E38" s="5">
-        <f>IF(AND(C38="yes",ISNUMBER(G38)),MAX(DATE(2026,5,11),G38),"")</f>
+        <f>IF(AND(C38="yes",ISNUMBER(G38)),MAX(DATE(2026,5,13),G38),"")</f>
         <v/>
       </c>
       <c r="F38" s="5">
@@ -4056,7 +4056,7 @@
         <v/>
       </c>
       <c r="E39" s="5">
-        <f>IF(AND(C39="yes",ISNUMBER(G39)),MAX(DATE(2026,5,11),G39),"")</f>
+        <f>IF(AND(C39="yes",ISNUMBER(G39)),MAX(DATE(2026,5,13),G39),"")</f>
         <v/>
       </c>
       <c r="F39" s="5">
@@ -4147,7 +4147,7 @@
         <v/>
       </c>
       <c r="E40" s="5">
-        <f>IF(AND(C40="yes",ISNUMBER(G40)),MAX(DATE(2026,5,11),G40),"")</f>
+        <f>IF(AND(C40="yes",ISNUMBER(G40)),MAX(DATE(2026,5,13),G40),"")</f>
         <v/>
       </c>
       <c r="F40" s="5">
@@ -4238,7 +4238,7 @@
         <v/>
       </c>
       <c r="E41" s="5">
-        <f>IF(AND(C41="yes",ISNUMBER(G41)),MAX(DATE(2026,5,11),G41),"")</f>
+        <f>IF(AND(C41="yes",ISNUMBER(G41)),MAX(DATE(2026,5,13),G41),"")</f>
         <v/>
       </c>
       <c r="F41" s="5">
@@ -4329,7 +4329,7 @@
         <v/>
       </c>
       <c r="E42" s="5">
-        <f>IF(AND(C42="yes",ISNUMBER(G42)),MAX(DATE(2026,5,11),G42),"")</f>
+        <f>IF(AND(C42="yes",ISNUMBER(G42)),MAX(DATE(2026,5,13),G42),"")</f>
         <v/>
       </c>
       <c r="F42" s="5">
@@ -4420,7 +4420,7 @@
         <v/>
       </c>
       <c r="E43" s="5">
-        <f>IF(AND(C43="yes",ISNUMBER(G43)),MAX(DATE(2026,5,11),G43),"")</f>
+        <f>IF(AND(C43="yes",ISNUMBER(G43)),MAX(DATE(2026,5,13),G43),"")</f>
         <v/>
       </c>
       <c r="F43" s="5">
@@ -4511,7 +4511,7 @@
         <v/>
       </c>
       <c r="E44" s="5">
-        <f>IF(AND(C44="yes",ISNUMBER(G44)),MAX(DATE(2026,5,11),G44),"")</f>
+        <f>IF(AND(C44="yes",ISNUMBER(G44)),MAX(DATE(2026,5,13),G44),"")</f>
         <v/>
       </c>
       <c r="F44" s="5">
@@ -4602,7 +4602,7 @@
         <v/>
       </c>
       <c r="E45" s="5">
-        <f>IF(AND(C45="yes",ISNUMBER(G45)),MAX(DATE(2026,5,11),G45),"")</f>
+        <f>IF(AND(C45="yes",ISNUMBER(G45)),MAX(DATE(2026,5,13),G45),"")</f>
         <v/>
       </c>
       <c r="F45" s="5">
@@ -4693,7 +4693,7 @@
         <v/>
       </c>
       <c r="E46" s="5">
-        <f>IF(AND(C46="yes",ISNUMBER(G46)),MAX(DATE(2026,5,11),G46),"")</f>
+        <f>IF(AND(C46="yes",ISNUMBER(G46)),MAX(DATE(2026,5,13),G46),"")</f>
         <v/>
       </c>
       <c r="F46" s="5">
@@ -4784,7 +4784,7 @@
         <v/>
       </c>
       <c r="E47" s="5">
-        <f>IF(AND(C47="yes",ISNUMBER(G47)),MAX(DATE(2026,5,11),G47),"")</f>
+        <f>IF(AND(C47="yes",ISNUMBER(G47)),MAX(DATE(2026,5,13),G47),"")</f>
         <v/>
       </c>
       <c r="F47" s="5">
@@ -4875,7 +4875,7 @@
         <v/>
       </c>
       <c r="E48" s="5">
-        <f>IF(AND(C48="yes",ISNUMBER(G48)),MAX(DATE(2026,5,11),G48),"")</f>
+        <f>IF(AND(C48="yes",ISNUMBER(G48)),MAX(DATE(2026,5,13),G48),"")</f>
         <v/>
       </c>
       <c r="F48" s="5">
@@ -4966,7 +4966,7 @@
         <v/>
       </c>
       <c r="E49" s="5">
-        <f>IF(AND(C49="yes",ISNUMBER(G49)),MAX(DATE(2026,5,11),G49),"")</f>
+        <f>IF(AND(C49="yes",ISNUMBER(G49)),MAX(DATE(2026,5,13),G49),"")</f>
         <v/>
       </c>
       <c r="F49" s="5">
@@ -5057,7 +5057,7 @@
         <v/>
       </c>
       <c r="E50" s="5">
-        <f>IF(AND(C50="yes",ISNUMBER(G50)),MAX(DATE(2026,5,11),G50),"")</f>
+        <f>IF(AND(C50="yes",ISNUMBER(G50)),MAX(DATE(2026,5,13),G50),"")</f>
         <v/>
       </c>
       <c r="F50" s="5">
@@ -5148,7 +5148,7 @@
         <v/>
       </c>
       <c r="E51" s="5">
-        <f>IF(AND(C51="yes",ISNUMBER(G51)),MAX(DATE(2026,5,11),G51),"")</f>
+        <f>IF(AND(C51="yes",ISNUMBER(G51)),MAX(DATE(2026,5,13),G51),"")</f>
         <v/>
       </c>
       <c r="F51" s="5">
@@ -5239,7 +5239,7 @@
         <v/>
       </c>
       <c r="E52" s="5">
-        <f>IF(AND(C52="yes",ISNUMBER(G52)),MAX(DATE(2026,5,11),G52),"")</f>
+        <f>IF(AND(C52="yes",ISNUMBER(G52)),MAX(DATE(2026,5,13),G52),"")</f>
         <v/>
       </c>
       <c r="F52" s="5">
@@ -5330,7 +5330,7 @@
         <v/>
       </c>
       <c r="E53" s="5">
-        <f>IF(AND(C53="yes",ISNUMBER(G53)),MAX(DATE(2026,5,11),G53),"")</f>
+        <f>IF(AND(C53="yes",ISNUMBER(G53)),MAX(DATE(2026,5,13),G53),"")</f>
         <v/>
       </c>
       <c r="F53" s="5">
@@ -5421,7 +5421,7 @@
         <v/>
       </c>
       <c r="E54" s="5">
-        <f>IF(AND(C54="yes",ISNUMBER(G54)),MAX(DATE(2026,5,11),G54),"")</f>
+        <f>IF(AND(C54="yes",ISNUMBER(G54)),MAX(DATE(2026,5,13),G54),"")</f>
         <v/>
       </c>
       <c r="F54" s="5">
@@ -5512,7 +5512,7 @@
         <v/>
       </c>
       <c r="E55" s="5">
-        <f>IF(AND(C55="yes",ISNUMBER(G55)),MAX(DATE(2026,5,11),G55),"")</f>
+        <f>IF(AND(C55="yes",ISNUMBER(G55)),MAX(DATE(2026,5,13),G55),"")</f>
         <v/>
       </c>
       <c r="F55" s="5">
@@ -5603,7 +5603,7 @@
         <v/>
       </c>
       <c r="E56" s="5">
-        <f>IF(AND(C56="yes",ISNUMBER(G56)),MAX(DATE(2026,5,11),G56),"")</f>
+        <f>IF(AND(C56="yes",ISNUMBER(G56)),MAX(DATE(2026,5,13),G56),"")</f>
         <v/>
       </c>
       <c r="F56" s="5">
@@ -5694,7 +5694,7 @@
         <v/>
       </c>
       <c r="E57" s="5">
-        <f>IF(AND(C57="yes",ISNUMBER(G57)),MAX(DATE(2026,5,11),G57),"")</f>
+        <f>IF(AND(C57="yes",ISNUMBER(G57)),MAX(DATE(2026,5,13),G57),"")</f>
         <v/>
       </c>
       <c r="F57" s="5">
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="E58" s="5">
-        <f>IF(AND(C58="yes",ISNUMBER(G58)),MAX(DATE(2026,5,11),G58),"")</f>
+        <f>IF(AND(C58="yes",ISNUMBER(G58)),MAX(DATE(2026,5,13),G58),"")</f>
         <v/>
       </c>
       <c r="F58" s="5">
@@ -5876,7 +5876,7 @@
         <v/>
       </c>
       <c r="E59" s="5">
-        <f>IF(AND(C59="yes",ISNUMBER(G59)),MAX(DATE(2026,5,11),G59),"")</f>
+        <f>IF(AND(C59="yes",ISNUMBER(G59)),MAX(DATE(2026,5,13),G59),"")</f>
         <v/>
       </c>
       <c r="F59" s="5">
@@ -5967,7 +5967,7 @@
         <v/>
       </c>
       <c r="E60" s="5">
-        <f>IF(AND(C60="yes",ISNUMBER(G60)),MAX(DATE(2026,5,11),G60),"")</f>
+        <f>IF(AND(C60="yes",ISNUMBER(G60)),MAX(DATE(2026,5,13),G60),"")</f>
         <v/>
       </c>
       <c r="F60" s="5">
@@ -6058,7 +6058,7 @@
         <v/>
       </c>
       <c r="E61" s="5">
-        <f>IF(AND(C61="yes",ISNUMBER(G61)),MAX(DATE(2026,5,11),G61),"")</f>
+        <f>IF(AND(C61="yes",ISNUMBER(G61)),MAX(DATE(2026,5,13),G61),"")</f>
         <v/>
       </c>
       <c r="F61" s="5">
@@ -6149,7 +6149,7 @@
         <v/>
       </c>
       <c r="E62" s="5">
-        <f>IF(AND(C62="yes",ISNUMBER(G62)),MAX(DATE(2026,5,11),G62),"")</f>
+        <f>IF(AND(C62="yes",ISNUMBER(G62)),MAX(DATE(2026,5,13),G62),"")</f>
         <v/>
       </c>
       <c r="F62" s="5">
@@ -6240,7 +6240,7 @@
         <v/>
       </c>
       <c r="E63" s="5">
-        <f>IF(AND(C63="yes",ISNUMBER(G63)),MAX(DATE(2026,5,11),G63),"")</f>
+        <f>IF(AND(C63="yes",ISNUMBER(G63)),MAX(DATE(2026,5,13),G63),"")</f>
         <v/>
       </c>
       <c r="F63" s="5">
@@ -6331,7 +6331,7 @@
         <v/>
       </c>
       <c r="E64" s="5">
-        <f>IF(AND(C64="yes",ISNUMBER(G64)),MAX(DATE(2026,5,11),G64),"")</f>
+        <f>IF(AND(C64="yes",ISNUMBER(G64)),MAX(DATE(2026,5,13),G64),"")</f>
         <v/>
       </c>
       <c r="F64" s="5">
@@ -6422,7 +6422,7 @@
         <v/>
       </c>
       <c r="E65" s="5">
-        <f>IF(AND(C65="yes",ISNUMBER(G65)),MAX(DATE(2026,5,11),G65),"")</f>
+        <f>IF(AND(C65="yes",ISNUMBER(G65)),MAX(DATE(2026,5,13),G65),"")</f>
         <v/>
       </c>
       <c r="F65" s="5">
@@ -6513,7 +6513,7 @@
         <v/>
       </c>
       <c r="E66" s="5">
-        <f>IF(AND(C66="yes",ISNUMBER(G66)),MAX(DATE(2026,5,11),G66),"")</f>
+        <f>IF(AND(C66="yes",ISNUMBER(G66)),MAX(DATE(2026,5,13),G66),"")</f>
         <v/>
       </c>
       <c r="F66" s="5">
@@ -6604,7 +6604,7 @@
         <v/>
       </c>
       <c r="E67" s="5">
-        <f>IF(AND(C67="yes",ISNUMBER(G67)),MAX(DATE(2026,5,11),G67),"")</f>
+        <f>IF(AND(C67="yes",ISNUMBER(G67)),MAX(DATE(2026,5,13),G67),"")</f>
         <v/>
       </c>
       <c r="F67" s="5">
@@ -6695,7 +6695,7 @@
         <v/>
       </c>
       <c r="E68" s="5">
-        <f>IF(AND(C68="yes",ISNUMBER(G68)),MAX(DATE(2026,5,11),G68),"")</f>
+        <f>IF(AND(C68="yes",ISNUMBER(G68)),MAX(DATE(2026,5,13),G68),"")</f>
         <v/>
       </c>
       <c r="F68" s="5">
@@ -6786,7 +6786,7 @@
         <v/>
       </c>
       <c r="E69" s="5">
-        <f>IF(AND(C69="yes",ISNUMBER(G69)),MAX(DATE(2026,5,11),G69),"")</f>
+        <f>IF(AND(C69="yes",ISNUMBER(G69)),MAX(DATE(2026,5,13),G69),"")</f>
         <v/>
       </c>
       <c r="F69" s="5">
@@ -6877,7 +6877,7 @@
         <v/>
       </c>
       <c r="E70" s="5">
-        <f>IF(AND(C70="yes",ISNUMBER(G70)),MAX(DATE(2026,5,11),G70),"")</f>
+        <f>IF(AND(C70="yes",ISNUMBER(G70)),MAX(DATE(2026,5,13),G70),"")</f>
         <v/>
       </c>
       <c r="F70" s="5">
@@ -6968,7 +6968,7 @@
         <v/>
       </c>
       <c r="E71" s="5">
-        <f>IF(AND(C71="yes",ISNUMBER(G71)),MAX(DATE(2026,5,11),G71),"")</f>
+        <f>IF(AND(C71="yes",ISNUMBER(G71)),MAX(DATE(2026,5,13),G71),"")</f>
         <v/>
       </c>
       <c r="F71" s="5">
@@ -7059,7 +7059,7 @@
         <v/>
       </c>
       <c r="E72" s="5">
-        <f>IF(AND(C72="yes",ISNUMBER(G72)),MAX(DATE(2026,5,11),G72),"")</f>
+        <f>IF(AND(C72="yes",ISNUMBER(G72)),MAX(DATE(2026,5,13),G72),"")</f>
         <v/>
       </c>
       <c r="F72" s="5">
@@ -7150,7 +7150,7 @@
         <v/>
       </c>
       <c r="E73" s="5">
-        <f>IF(AND(C73="yes",ISNUMBER(G73)),MAX(DATE(2026,5,11),G73),"")</f>
+        <f>IF(AND(C73="yes",ISNUMBER(G73)),MAX(DATE(2026,5,13),G73),"")</f>
         <v/>
       </c>
       <c r="F73" s="5">
@@ -7241,7 +7241,7 @@
         <v/>
       </c>
       <c r="E74" s="5">
-        <f>IF(AND(C74="yes",ISNUMBER(G74)),MAX(DATE(2026,5,11),G74),"")</f>
+        <f>IF(AND(C74="yes",ISNUMBER(G74)),MAX(DATE(2026,5,13),G74),"")</f>
         <v/>
       </c>
       <c r="F74" s="5">
@@ -7332,7 +7332,7 @@
         <v/>
       </c>
       <c r="E75" s="5">
-        <f>IF(AND(C75="yes",ISNUMBER(G75)),MAX(DATE(2026,5,11),G75),"")</f>
+        <f>IF(AND(C75="yes",ISNUMBER(G75)),MAX(DATE(2026,5,13),G75),"")</f>
         <v/>
       </c>
       <c r="F75" s="5">
@@ -7423,7 +7423,7 @@
         <v/>
       </c>
       <c r="E76" s="5">
-        <f>IF(AND(C76="yes",ISNUMBER(G76)),MAX(DATE(2026,5,11),G76),"")</f>
+        <f>IF(AND(C76="yes",ISNUMBER(G76)),MAX(DATE(2026,5,13),G76),"")</f>
         <v/>
       </c>
       <c r="F76" s="5">
@@ -7514,7 +7514,7 @@
         <v/>
       </c>
       <c r="E77" s="5">
-        <f>IF(AND(C77="yes",ISNUMBER(G77)),MAX(DATE(2026,5,11),G77),"")</f>
+        <f>IF(AND(C77="yes",ISNUMBER(G77)),MAX(DATE(2026,5,13),G77),"")</f>
         <v/>
       </c>
       <c r="F77" s="5">
@@ -7605,7 +7605,7 @@
         <v/>
       </c>
       <c r="E78" s="5">
-        <f>IF(AND(C78="yes",ISNUMBER(G78)),MAX(DATE(2026,5,11),G78),"")</f>
+        <f>IF(AND(C78="yes",ISNUMBER(G78)),MAX(DATE(2026,5,13),G78),"")</f>
         <v/>
       </c>
       <c r="F78" s="5">
@@ -7696,7 +7696,7 @@
         <v/>
       </c>
       <c r="E79" s="5">
-        <f>IF(AND(C79="yes",ISNUMBER(G79)),MAX(DATE(2026,5,11),G79),"")</f>
+        <f>IF(AND(C79="yes",ISNUMBER(G79)),MAX(DATE(2026,5,13),G79),"")</f>
         <v/>
       </c>
       <c r="F79" s="5">
@@ -7787,7 +7787,7 @@
         <v/>
       </c>
       <c r="E80" s="5">
-        <f>IF(AND(C80="yes",ISNUMBER(G80)),MAX(DATE(2026,5,11),G80),"")</f>
+        <f>IF(AND(C80="yes",ISNUMBER(G80)),MAX(DATE(2026,5,13),G80),"")</f>
         <v/>
       </c>
       <c r="F80" s="5">
@@ -7878,7 +7878,7 @@
         <v/>
       </c>
       <c r="E81" s="5">
-        <f>IF(AND(C81="yes",ISNUMBER(G81)),MAX(DATE(2026,5,11),G81),"")</f>
+        <f>IF(AND(C81="yes",ISNUMBER(G81)),MAX(DATE(2026,5,13),G81),"")</f>
         <v/>
       </c>
       <c r="F81" s="5">
@@ -7969,7 +7969,7 @@
         <v/>
       </c>
       <c r="E82" s="5">
-        <f>IF(AND(C82="yes",ISNUMBER(G82)),MAX(DATE(2026,5,11),G82),"")</f>
+        <f>IF(AND(C82="yes",ISNUMBER(G82)),MAX(DATE(2026,5,13),G82),"")</f>
         <v/>
       </c>
       <c r="F82" s="5">
@@ -8060,7 +8060,7 @@
         <v/>
       </c>
       <c r="E83" s="5">
-        <f>IF(AND(C83="yes",ISNUMBER(G83)),MAX(DATE(2026,5,11),G83),"")</f>
+        <f>IF(AND(C83="yes",ISNUMBER(G83)),MAX(DATE(2026,5,13),G83),"")</f>
         <v/>
       </c>
       <c r="F83" s="5">
@@ -8151,7 +8151,7 @@
         <v/>
       </c>
       <c r="E84" s="5">
-        <f>IF(AND(C84="yes",ISNUMBER(G84)),MAX(DATE(2026,5,11),G84),"")</f>
+        <f>IF(AND(C84="yes",ISNUMBER(G84)),MAX(DATE(2026,5,13),G84),"")</f>
         <v/>
       </c>
       <c r="F84" s="5">
@@ -8242,7 +8242,7 @@
         <v/>
       </c>
       <c r="E85" s="5">
-        <f>IF(AND(C85="yes",ISNUMBER(G85)),MAX(DATE(2026,5,11),G85),"")</f>
+        <f>IF(AND(C85="yes",ISNUMBER(G85)),MAX(DATE(2026,5,13),G85),"")</f>
         <v/>
       </c>
       <c r="F85" s="5">
@@ -8333,7 +8333,7 @@
         <v/>
       </c>
       <c r="E86" s="5">
-        <f>IF(AND(C86="yes",ISNUMBER(G86)),MAX(DATE(2026,5,11),G86),"")</f>
+        <f>IF(AND(C86="yes",ISNUMBER(G86)),MAX(DATE(2026,5,13),G86),"")</f>
         <v/>
       </c>
       <c r="F86" s="5">
@@ -8424,7 +8424,7 @@
         <v/>
       </c>
       <c r="E87" s="5">
-        <f>IF(AND(C87="yes",ISNUMBER(G87)),MAX(DATE(2026,5,11),G87),"")</f>
+        <f>IF(AND(C87="yes",ISNUMBER(G87)),MAX(DATE(2026,5,13),G87),"")</f>
         <v/>
       </c>
       <c r="F87" s="5">
@@ -8515,7 +8515,7 @@
         <v/>
       </c>
       <c r="E88" s="5">
-        <f>IF(AND(C88="yes",ISNUMBER(G88)),MAX(DATE(2026,5,11),G88),"")</f>
+        <f>IF(AND(C88="yes",ISNUMBER(G88)),MAX(DATE(2026,5,13),G88),"")</f>
         <v/>
       </c>
       <c r="F88" s="5">
@@ -8602,7 +8602,7 @@
         <v/>
       </c>
       <c r="E89" s="5">
-        <f>IF(AND(C89="yes",ISNUMBER(G89)),MAX(DATE(2026,5,11),G89),"")</f>
+        <f>IF(AND(C89="yes",ISNUMBER(G89)),MAX(DATE(2026,5,13),G89),"")</f>
         <v/>
       </c>
       <c r="F89" s="5">
@@ -8689,7 +8689,7 @@
         <v/>
       </c>
       <c r="E90" s="5">
-        <f>IF(AND(C90="yes",ISNUMBER(G90)),MAX(DATE(2026,5,11),G90),"")</f>
+        <f>IF(AND(C90="yes",ISNUMBER(G90)),MAX(DATE(2026,5,13),G90),"")</f>
         <v/>
       </c>
       <c r="F90" s="5">
@@ -8780,7 +8780,7 @@
         <v/>
       </c>
       <c r="E91" s="5">
-        <f>IF(AND(C91="yes",ISNUMBER(G91)),MAX(DATE(2026,5,11),G91),"")</f>
+        <f>IF(AND(C91="yes",ISNUMBER(G91)),MAX(DATE(2026,5,13),G91),"")</f>
         <v/>
       </c>
       <c r="F91" s="5">
@@ -8871,7 +8871,7 @@
         <v/>
       </c>
       <c r="E92" s="5">
-        <f>IF(AND(C92="yes",ISNUMBER(G92)),MAX(DATE(2026,5,11),G92),"")</f>
+        <f>IF(AND(C92="yes",ISNUMBER(G92)),MAX(DATE(2026,5,13),G92),"")</f>
         <v/>
       </c>
       <c r="F92" s="5">
@@ -8962,7 +8962,7 @@
         <v/>
       </c>
       <c r="E93" s="5">
-        <f>IF(AND(C93="yes",ISNUMBER(G93)),MAX(DATE(2026,5,11),G93),"")</f>
+        <f>IF(AND(C93="yes",ISNUMBER(G93)),MAX(DATE(2026,5,13),G93),"")</f>
         <v/>
       </c>
       <c r="F93" s="5">
@@ -9053,7 +9053,7 @@
         <v/>
       </c>
       <c r="E94" s="5">
-        <f>IF(AND(C94="yes",ISNUMBER(G94)),MAX(DATE(2026,5,11),G94),"")</f>
+        <f>IF(AND(C94="yes",ISNUMBER(G94)),MAX(DATE(2026,5,13),G94),"")</f>
         <v/>
       </c>
       <c r="F94" s="5">
@@ -9144,7 +9144,7 @@
         <v/>
       </c>
       <c r="E95" s="5">
-        <f>IF(AND(C95="yes",ISNUMBER(G95)),MAX(DATE(2026,5,11),G95),"")</f>
+        <f>IF(AND(C95="yes",ISNUMBER(G95)),MAX(DATE(2026,5,13),G95),"")</f>
         <v/>
       </c>
       <c r="F95" s="5">
@@ -9235,7 +9235,7 @@
         <v/>
       </c>
       <c r="E96" s="5">
-        <f>IF(AND(C96="yes",ISNUMBER(G96)),MAX(DATE(2026,5,11),G96),"")</f>
+        <f>IF(AND(C96="yes",ISNUMBER(G96)),MAX(DATE(2026,5,13),G96),"")</f>
         <v/>
       </c>
       <c r="F96" s="5">
@@ -9326,7 +9326,7 @@
         <v/>
       </c>
       <c r="E97" s="5">
-        <f>IF(AND(C97="yes",ISNUMBER(G97)),MAX(DATE(2026,5,11),G97),"")</f>
+        <f>IF(AND(C97="yes",ISNUMBER(G97)),MAX(DATE(2026,5,13),G97),"")</f>
         <v/>
       </c>
       <c r="F97" s="5">
@@ -9417,7 +9417,7 @@
         <v/>
       </c>
       <c r="E98" s="5">
-        <f>IF(AND(C98="yes",ISNUMBER(G98)),MAX(DATE(2026,5,11),G98),"")</f>
+        <f>IF(AND(C98="yes",ISNUMBER(G98)),MAX(DATE(2026,5,13),G98),"")</f>
         <v/>
       </c>
       <c r="F98" s="5">
@@ -9508,7 +9508,7 @@
         <v/>
       </c>
       <c r="E99" s="5">
-        <f>IF(AND(C99="yes",ISNUMBER(G99)),MAX(DATE(2026,5,11),G99),"")</f>
+        <f>IF(AND(C99="yes",ISNUMBER(G99)),MAX(DATE(2026,5,13),G99),"")</f>
         <v/>
       </c>
       <c r="F99" s="5">
@@ -9599,7 +9599,7 @@
         <v/>
       </c>
       <c r="E100" s="5">
-        <f>IF(AND(C100="yes",ISNUMBER(G100)),MAX(DATE(2026,5,11),G100),"")</f>
+        <f>IF(AND(C100="yes",ISNUMBER(G100)),MAX(DATE(2026,5,13),G100),"")</f>
         <v/>
       </c>
       <c r="F100" s="5">
@@ -9690,7 +9690,7 @@
         <v/>
       </c>
       <c r="E101" s="5">
-        <f>IF(AND(C101="yes",ISNUMBER(G101)),MAX(DATE(2026,5,11),G101),"")</f>
+        <f>IF(AND(C101="yes",ISNUMBER(G101)),MAX(DATE(2026,5,13),G101),"")</f>
         <v/>
       </c>
       <c r="F101" s="5">
@@ -9781,7 +9781,7 @@
         <v/>
       </c>
       <c r="E102" s="5">
-        <f>IF(AND(C102="yes",ISNUMBER(G102)),MAX(DATE(2026,5,11),G102),"")</f>
+        <f>IF(AND(C102="yes",ISNUMBER(G102)),MAX(DATE(2026,5,13),G102),"")</f>
         <v/>
       </c>
       <c r="F102" s="5">
@@ -9872,7 +9872,7 @@
         <v/>
       </c>
       <c r="E103" s="5">
-        <f>IF(AND(C103="yes",ISNUMBER(G103)),MAX(DATE(2026,5,11),G103),"")</f>
+        <f>IF(AND(C103="yes",ISNUMBER(G103)),MAX(DATE(2026,5,13),G103),"")</f>
         <v/>
       </c>
       <c r="F103" s="5">
@@ -9963,7 +9963,7 @@
         <v/>
       </c>
       <c r="E104" s="5">
-        <f>IF(AND(C104="yes",ISNUMBER(G104)),MAX(DATE(2026,5,11),G104),"")</f>
+        <f>IF(AND(C104="yes",ISNUMBER(G104)),MAX(DATE(2026,5,13),G104),"")</f>
         <v/>
       </c>
       <c r="F104" s="5">
@@ -10054,7 +10054,7 @@
         <v/>
       </c>
       <c r="E105" s="5">
-        <f>IF(AND(C105="yes",ISNUMBER(G105)),MAX(DATE(2026,5,11),G105),"")</f>
+        <f>IF(AND(C105="yes",ISNUMBER(G105)),MAX(DATE(2026,5,13),G105),"")</f>
         <v/>
       </c>
       <c r="F105" s="5">
@@ -10145,7 +10145,7 @@
         <v/>
       </c>
       <c r="E106" s="5">
-        <f>IF(AND(C106="yes",ISNUMBER(G106)),MAX(DATE(2026,5,11),G106),"")</f>
+        <f>IF(AND(C106="yes",ISNUMBER(G106)),MAX(DATE(2026,5,13),G106),"")</f>
         <v/>
       </c>
       <c r="F106" s="5">
@@ -10236,7 +10236,7 @@
         <v/>
       </c>
       <c r="E107" s="5">
-        <f>IF(AND(C107="yes",ISNUMBER(G107)),MAX(DATE(2026,5,11),G107),"")</f>
+        <f>IF(AND(C107="yes",ISNUMBER(G107)),MAX(DATE(2026,5,13),G107),"")</f>
         <v/>
       </c>
       <c r="F107" s="5">
@@ -10327,7 +10327,7 @@
         <v/>
       </c>
       <c r="E108" s="5">
-        <f>IF(AND(C108="yes",ISNUMBER(G108)),MAX(DATE(2026,5,11),G108),"")</f>
+        <f>IF(AND(C108="yes",ISNUMBER(G108)),MAX(DATE(2026,5,13),G108),"")</f>
         <v/>
       </c>
       <c r="F108" s="5">
@@ -10418,7 +10418,7 @@
         <v/>
       </c>
       <c r="E109" s="5">
-        <f>IF(AND(C109="yes",ISNUMBER(G109)),MAX(DATE(2026,5,11),G109),"")</f>
+        <f>IF(AND(C109="yes",ISNUMBER(G109)),MAX(DATE(2026,5,13),G109),"")</f>
         <v/>
       </c>
       <c r="F109" s="5">
@@ -10509,7 +10509,7 @@
         <v/>
       </c>
       <c r="E110" s="5">
-        <f>IF(AND(C110="yes",ISNUMBER(G110)),MAX(DATE(2026,5,11),G110),"")</f>
+        <f>IF(AND(C110="yes",ISNUMBER(G110)),MAX(DATE(2026,5,13),G110),"")</f>
         <v/>
       </c>
       <c r="F110" s="5">
@@ -10532,7 +10532,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>N/A — no P batch assigned</t>
+          <t>P060212</t>
         </is>
       </c>
       <c r="K110" s="2" t="inlineStr">
@@ -10600,7 +10600,7 @@
         <v/>
       </c>
       <c r="E111" s="5">
-        <f>IF(AND(C111="yes",ISNUMBER(G111)),MAX(DATE(2026,5,11),G111),"")</f>
+        <f>IF(AND(C111="yes",ISNUMBER(G111)),MAX(DATE(2026,5,13),G111),"")</f>
         <v/>
       </c>
       <c r="F111" s="5">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="J111" s="2" t="inlineStr">
         <is>
-          <t>N/A — no P batch assigned</t>
+          <t>P060212</t>
         </is>
       </c>
       <c r="K111" s="2" t="inlineStr">
@@ -10691,7 +10691,7 @@
         <v/>
       </c>
       <c r="E112" s="5">
-        <f>IF(AND(C112="yes",ISNUMBER(G112)),MAX(DATE(2026,5,11),G112),"")</f>
+        <f>IF(AND(C112="yes",ISNUMBER(G112)),MAX(DATE(2026,5,13),G112),"")</f>
         <v/>
       </c>
       <c r="F112" s="5">
@@ -10782,7 +10782,7 @@
         <v/>
       </c>
       <c r="E113" s="5">
-        <f>IF(AND(C113="yes",ISNUMBER(G113)),MAX(DATE(2026,5,11),G113),"")</f>
+        <f>IF(AND(C113="yes",ISNUMBER(G113)),MAX(DATE(2026,5,13),G113),"")</f>
         <v/>
       </c>
       <c r="F113" s="5">
@@ -10873,7 +10873,7 @@
         <v/>
       </c>
       <c r="E114" s="5">
-        <f>IF(AND(C114="yes",ISNUMBER(G114)),MAX(DATE(2026,5,11),G114),"")</f>
+        <f>IF(AND(C114="yes",ISNUMBER(G114)),MAX(DATE(2026,5,13),G114),"")</f>
         <v/>
       </c>
       <c r="F114" s="5">
@@ -10964,7 +10964,7 @@
         <v/>
       </c>
       <c r="E115" s="5">
-        <f>IF(AND(C115="yes",ISNUMBER(G115)),MAX(DATE(2026,5,11),G115),"")</f>
+        <f>IF(AND(C115="yes",ISNUMBER(G115)),MAX(DATE(2026,5,13),G115),"")</f>
         <v/>
       </c>
       <c r="F115" s="5">
@@ -11055,7 +11055,7 @@
         <v/>
       </c>
       <c r="E116" s="5">
-        <f>IF(AND(C116="yes",ISNUMBER(G116)),MAX(DATE(2026,5,11),G116),"")</f>
+        <f>IF(AND(C116="yes",ISNUMBER(G116)),MAX(DATE(2026,5,13),G116),"")</f>
         <v/>
       </c>
       <c r="F116" s="5">
@@ -11146,7 +11146,7 @@
         <v/>
       </c>
       <c r="E117" s="5">
-        <f>IF(AND(C117="yes",ISNUMBER(G117)),MAX(DATE(2026,5,11),G117),"")</f>
+        <f>IF(AND(C117="yes",ISNUMBER(G117)),MAX(DATE(2026,5,13),G117),"")</f>
         <v/>
       </c>
       <c r="F117" s="5">
@@ -11237,7 +11237,7 @@
         <v/>
       </c>
       <c r="E118" s="5">
-        <f>IF(AND(C118="yes",ISNUMBER(G118)),MAX(DATE(2026,5,11),G118),"")</f>
+        <f>IF(AND(C118="yes",ISNUMBER(G118)),MAX(DATE(2026,5,13),G118),"")</f>
         <v/>
       </c>
       <c r="F118" s="5">
@@ -11328,7 +11328,7 @@
         <v/>
       </c>
       <c r="E119" s="5">
-        <f>IF(AND(C119="yes",ISNUMBER(G119)),MAX(DATE(2026,5,11),G119),"")</f>
+        <f>IF(AND(C119="yes",ISNUMBER(G119)),MAX(DATE(2026,5,13),G119),"")</f>
         <v/>
       </c>
       <c r="F119" s="5">
@@ -11419,7 +11419,7 @@
         <v/>
       </c>
       <c r="E120" s="5">
-        <f>IF(AND(C120="yes",ISNUMBER(G120)),MAX(DATE(2026,5,11),G120),"")</f>
+        <f>IF(AND(C120="yes",ISNUMBER(G120)),MAX(DATE(2026,5,13),G120),"")</f>
         <v/>
       </c>
       <c r="F120" s="5">
@@ -11510,7 +11510,7 @@
         <v/>
       </c>
       <c r="E121" s="5">
-        <f>IF(AND(C121="yes",ISNUMBER(G121)),MAX(DATE(2026,5,11),G121),"")</f>
+        <f>IF(AND(C121="yes",ISNUMBER(G121)),MAX(DATE(2026,5,13),G121),"")</f>
         <v/>
       </c>
       <c r="F121" s="5">
@@ -11601,7 +11601,7 @@
         <v/>
       </c>
       <c r="E122" s="5">
-        <f>IF(AND(C122="yes",ISNUMBER(G122)),MAX(DATE(2026,5,11),G122),"")</f>
+        <f>IF(AND(C122="yes",ISNUMBER(G122)),MAX(DATE(2026,5,13),G122),"")</f>
         <v/>
       </c>
       <c r="F122" s="5">
@@ -11692,7 +11692,7 @@
         <v/>
       </c>
       <c r="E123" s="5">
-        <f>IF(AND(C123="yes",ISNUMBER(G123)),MAX(DATE(2026,5,11),G123),"")</f>
+        <f>IF(AND(C123="yes",ISNUMBER(G123)),MAX(DATE(2026,5,13),G123),"")</f>
         <v/>
       </c>
       <c r="F123" s="5">
@@ -11783,7 +11783,7 @@
         <v/>
       </c>
       <c r="E124" s="5">
-        <f>IF(AND(C124="yes",ISNUMBER(G124)),MAX(DATE(2026,5,11),G124),"")</f>
+        <f>IF(AND(C124="yes",ISNUMBER(G124)),MAX(DATE(2026,5,13),G124),"")</f>
         <v/>
       </c>
       <c r="F124" s="5">
@@ -11874,7 +11874,7 @@
         <v/>
       </c>
       <c r="E125" s="5">
-        <f>IF(AND(C125="yes",ISNUMBER(G125)),MAX(DATE(2026,5,11),G125),"")</f>
+        <f>IF(AND(C125="yes",ISNUMBER(G125)),MAX(DATE(2026,5,13),G125),"")</f>
         <v/>
       </c>
       <c r="F125" s="5">
@@ -11965,7 +11965,7 @@
         <v/>
       </c>
       <c r="E126" s="5">
-        <f>IF(AND(C126="yes",ISNUMBER(G126)),MAX(DATE(2026,5,11),G126),"")</f>
+        <f>IF(AND(C126="yes",ISNUMBER(G126)),MAX(DATE(2026,5,13),G126),"")</f>
         <v/>
       </c>
       <c r="F126" s="5">
@@ -12056,7 +12056,7 @@
         <v/>
       </c>
       <c r="E127" s="5">
-        <f>IF(AND(C127="yes",ISNUMBER(G127)),MAX(DATE(2026,5,11),G127),"")</f>
+        <f>IF(AND(C127="yes",ISNUMBER(G127)),MAX(DATE(2026,5,13),G127),"")</f>
         <v/>
       </c>
       <c r="F127" s="5">
@@ -12147,7 +12147,7 @@
         <v/>
       </c>
       <c r="E128" s="5">
-        <f>IF(AND(C128="yes",ISNUMBER(G128)),MAX(DATE(2026,5,11),G128),"")</f>
+        <f>IF(AND(C128="yes",ISNUMBER(G128)),MAX(DATE(2026,5,13),G128),"")</f>
         <v/>
       </c>
       <c r="F128" s="5">
@@ -12238,7 +12238,7 @@
         <v/>
       </c>
       <c r="E129" s="5">
-        <f>IF(AND(C129="yes",ISNUMBER(G129)),MAX(DATE(2026,5,11),G129),"")</f>
+        <f>IF(AND(C129="yes",ISNUMBER(G129)),MAX(DATE(2026,5,13),G129),"")</f>
         <v/>
       </c>
       <c r="F129" s="5">
@@ -12329,7 +12329,7 @@
         <v/>
       </c>
       <c r="E130" s="5">
-        <f>IF(AND(C130="yes",ISNUMBER(G130)),MAX(DATE(2026,5,11),G130),"")</f>
+        <f>IF(AND(C130="yes",ISNUMBER(G130)),MAX(DATE(2026,5,13),G130),"")</f>
         <v/>
       </c>
       <c r="F130" s="5">
@@ -12420,7 +12420,7 @@
         <v/>
       </c>
       <c r="E131" s="5">
-        <f>IF(AND(C131="yes",ISNUMBER(G131)),MAX(DATE(2026,5,11),G131),"")</f>
+        <f>IF(AND(C131="yes",ISNUMBER(G131)),MAX(DATE(2026,5,13),G131),"")</f>
         <v/>
       </c>
       <c r="F131" s="5">
@@ -12511,7 +12511,7 @@
         <v/>
       </c>
       <c r="E132" s="5">
-        <f>IF(AND(C132="yes",ISNUMBER(G132)),MAX(DATE(2026,5,11),G132),"")</f>
+        <f>IF(AND(C132="yes",ISNUMBER(G132)),MAX(DATE(2026,5,13),G132),"")</f>
         <v/>
       </c>
       <c r="F132" s="5">
@@ -12598,7 +12598,7 @@
         <v/>
       </c>
       <c r="E133" s="5">
-        <f>IF(AND(C133="yes",ISNUMBER(G133)),MAX(DATE(2026,5,11),G133),"")</f>
+        <f>IF(AND(C133="yes",ISNUMBER(G133)),MAX(DATE(2026,5,13),G133),"")</f>
         <v/>
       </c>
       <c r="F133" s="5">
@@ -12685,7 +12685,7 @@
         <v/>
       </c>
       <c r="E134" s="5">
-        <f>IF(AND(C134="yes",ISNUMBER(G134)),MAX(DATE(2026,5,11),G134),"")</f>
+        <f>IF(AND(C134="yes",ISNUMBER(G134)),MAX(DATE(2026,5,13),G134),"")</f>
         <v/>
       </c>
       <c r="F134" s="5">
@@ -12776,7 +12776,7 @@
         <v/>
       </c>
       <c r="E135" s="5">
-        <f>IF(AND(C135="yes",ISNUMBER(G135)),MAX(DATE(2026,5,11),G135),"")</f>
+        <f>IF(AND(C135="yes",ISNUMBER(G135)),MAX(DATE(2026,5,13),G135),"")</f>
         <v/>
       </c>
       <c r="F135" s="5">
@@ -12867,7 +12867,7 @@
         <v/>
       </c>
       <c r="E136" s="5">
-        <f>IF(AND(C136="yes",ISNUMBER(G136)),MAX(DATE(2026,5,11),G136),"")</f>
+        <f>IF(AND(C136="yes",ISNUMBER(G136)),MAX(DATE(2026,5,13),G136),"")</f>
         <v/>
       </c>
       <c r="F136" s="5">
@@ -12958,7 +12958,7 @@
         <v/>
       </c>
       <c r="E137" s="5">
-        <f>IF(AND(C137="yes",ISNUMBER(G137)),MAX(DATE(2026,5,11),G137),"")</f>
+        <f>IF(AND(C137="yes",ISNUMBER(G137)),MAX(DATE(2026,5,13),G137),"")</f>
         <v/>
       </c>
       <c r="F137" s="5">
@@ -13049,7 +13049,7 @@
         <v/>
       </c>
       <c r="E138" s="5">
-        <f>IF(AND(C138="yes",ISNUMBER(G138)),MAX(DATE(2026,5,11),G138),"")</f>
+        <f>IF(AND(C138="yes",ISNUMBER(G138)),MAX(DATE(2026,5,13),G138),"")</f>
         <v/>
       </c>
       <c r="F138" s="5">
@@ -13140,7 +13140,7 @@
         <v/>
       </c>
       <c r="E139" s="5">
-        <f>IF(AND(C139="yes",ISNUMBER(G139)),MAX(DATE(2026,5,11),G139),"")</f>
+        <f>IF(AND(C139="yes",ISNUMBER(G139)),MAX(DATE(2026,5,13),G139),"")</f>
         <v/>
       </c>
       <c r="F139" s="5">
@@ -13231,7 +13231,7 @@
         <v/>
       </c>
       <c r="E140" s="5">
-        <f>IF(AND(C140="yes",ISNUMBER(G140)),MAX(DATE(2026,5,11),G140),"")</f>
+        <f>IF(AND(C140="yes",ISNUMBER(G140)),MAX(DATE(2026,5,13),G140),"")</f>
         <v/>
       </c>
       <c r="F140" s="5">
@@ -13322,7 +13322,7 @@
         <v/>
       </c>
       <c r="E141" s="5">
-        <f>IF(AND(C141="yes",ISNUMBER(G141)),MAX(DATE(2026,5,11),G141),"")</f>
+        <f>IF(AND(C141="yes",ISNUMBER(G141)),MAX(DATE(2026,5,13),G141),"")</f>
         <v/>
       </c>
       <c r="F141" s="5">
@@ -13413,7 +13413,7 @@
         <v/>
       </c>
       <c r="E142" s="5">
-        <f>IF(AND(C142="yes",ISNUMBER(G142)),MAX(DATE(2026,5,11),G142),"")</f>
+        <f>IF(AND(C142="yes",ISNUMBER(G142)),MAX(DATE(2026,5,13),G142),"")</f>
         <v/>
       </c>
       <c r="F142" s="5">
@@ -13504,7 +13504,7 @@
         <v/>
       </c>
       <c r="E143" s="5">
-        <f>IF(AND(C143="yes",ISNUMBER(G143)),MAX(DATE(2026,5,11),G143),"")</f>
+        <f>IF(AND(C143="yes",ISNUMBER(G143)),MAX(DATE(2026,5,13),G143),"")</f>
         <v/>
       </c>
       <c r="F143" s="5">
@@ -13595,7 +13595,7 @@
         <v/>
       </c>
       <c r="E144" s="5">
-        <f>IF(AND(C144="yes",ISNUMBER(G144)),MAX(DATE(2026,5,11),G144),"")</f>
+        <f>IF(AND(C144="yes",ISNUMBER(G144)),MAX(DATE(2026,5,13),G144),"")</f>
         <v/>
       </c>
       <c r="F144" s="5">
@@ -13686,7 +13686,7 @@
         <v/>
       </c>
       <c r="E145" s="5">
-        <f>IF(AND(C145="yes",ISNUMBER(G145)),MAX(DATE(2026,5,11),G145),"")</f>
+        <f>IF(AND(C145="yes",ISNUMBER(G145)),MAX(DATE(2026,5,13),G145),"")</f>
         <v/>
       </c>
       <c r="F145" s="5">
@@ -13777,7 +13777,7 @@
         <v/>
       </c>
       <c r="E146" s="5">
-        <f>IF(AND(C146="yes",ISNUMBER(G146)),MAX(DATE(2026,5,11),G146),"")</f>
+        <f>IF(AND(C146="yes",ISNUMBER(G146)),MAX(DATE(2026,5,13),G146),"")</f>
         <v/>
       </c>
       <c r="F146" s="5">
@@ -13868,7 +13868,7 @@
         <v/>
       </c>
       <c r="E147" s="5">
-        <f>IF(AND(C147="yes",ISNUMBER(G147)),MAX(DATE(2026,5,11),G147),"")</f>
+        <f>IF(AND(C147="yes",ISNUMBER(G147)),MAX(DATE(2026,5,13),G147),"")</f>
         <v/>
       </c>
       <c r="F147" s="5">
@@ -13959,7 +13959,7 @@
         <v/>
       </c>
       <c r="E148" s="5">
-        <f>IF(AND(C148="yes",ISNUMBER(G148)),MAX(DATE(2026,5,11),G148),"")</f>
+        <f>IF(AND(C148="yes",ISNUMBER(G148)),MAX(DATE(2026,5,13),G148),"")</f>
         <v/>
       </c>
       <c r="F148" s="5">
@@ -14050,7 +14050,7 @@
         <v/>
       </c>
       <c r="E149" s="5">
-        <f>IF(AND(C149="yes",ISNUMBER(G149)),MAX(DATE(2026,5,11),G149),"")</f>
+        <f>IF(AND(C149="yes",ISNUMBER(G149)),MAX(DATE(2026,5,13),G149),"")</f>
         <v/>
       </c>
       <c r="F149" s="5">
@@ -14141,7 +14141,7 @@
         <v/>
       </c>
       <c r="E150" s="5">
-        <f>IF(AND(C150="yes",ISNUMBER(G150)),MAX(DATE(2026,5,11),G150),"")</f>
+        <f>IF(AND(C150="yes",ISNUMBER(G150)),MAX(DATE(2026,5,13),G150),"")</f>
         <v/>
       </c>
       <c r="F150" s="5">
@@ -14232,7 +14232,7 @@
         <v/>
       </c>
       <c r="E151" s="5">
-        <f>IF(AND(C151="yes",ISNUMBER(G151)),MAX(DATE(2026,5,11),G151),"")</f>
+        <f>IF(AND(C151="yes",ISNUMBER(G151)),MAX(DATE(2026,5,13),G151),"")</f>
         <v/>
       </c>
       <c r="F151" s="5">
@@ -14323,7 +14323,7 @@
         <v/>
       </c>
       <c r="E152" s="5">
-        <f>IF(AND(C152="yes",ISNUMBER(G152)),MAX(DATE(2026,5,11),G152),"")</f>
+        <f>IF(AND(C152="yes",ISNUMBER(G152)),MAX(DATE(2026,5,13),G152),"")</f>
         <v/>
       </c>
       <c r="F152" s="5">
@@ -14414,7 +14414,7 @@
         <v/>
       </c>
       <c r="E153" s="5">
-        <f>IF(AND(C153="yes",ISNUMBER(G153)),MAX(DATE(2026,5,11),G153),"")</f>
+        <f>IF(AND(C153="yes",ISNUMBER(G153)),MAX(DATE(2026,5,13),G153),"")</f>
         <v/>
       </c>
       <c r="F153" s="5">
@@ -14505,7 +14505,7 @@
         <v/>
       </c>
       <c r="E154" s="5">
-        <f>IF(AND(C154="yes",ISNUMBER(G154)),MAX(DATE(2026,5,11),G154),"")</f>
+        <f>IF(AND(C154="yes",ISNUMBER(G154)),MAX(DATE(2026,5,13),G154),"")</f>
         <v/>
       </c>
       <c r="F154" s="5">
@@ -14596,7 +14596,7 @@
         <v/>
       </c>
       <c r="E155" s="5">
-        <f>IF(AND(C155="yes",ISNUMBER(G155)),MAX(DATE(2026,5,11),G155),"")</f>
+        <f>IF(AND(C155="yes",ISNUMBER(G155)),MAX(DATE(2026,5,13),G155),"")</f>
         <v/>
       </c>
       <c r="F155" s="5">
@@ -14687,7 +14687,7 @@
         <v/>
       </c>
       <c r="E156" s="5">
-        <f>IF(AND(C156="yes",ISNUMBER(G156)),MAX(DATE(2026,5,11),G156),"")</f>
+        <f>IF(AND(C156="yes",ISNUMBER(G156)),MAX(DATE(2026,5,13),G156),"")</f>
         <v/>
       </c>
       <c r="F156" s="5">
@@ -14778,7 +14778,7 @@
         <v/>
       </c>
       <c r="E157" s="5">
-        <f>IF(AND(C157="yes",ISNUMBER(G157)),MAX(DATE(2026,5,11),G157),"")</f>
+        <f>IF(AND(C157="yes",ISNUMBER(G157)),MAX(DATE(2026,5,13),G157),"")</f>
         <v/>
       </c>
       <c r="F157" s="5">
@@ -14869,7 +14869,7 @@
         <v/>
       </c>
       <c r="E158" s="5">
-        <f>IF(AND(C158="yes",ISNUMBER(G158)),MAX(DATE(2026,5,11),G158),"")</f>
+        <f>IF(AND(C158="yes",ISNUMBER(G158)),MAX(DATE(2026,5,13),G158),"")</f>
         <v/>
       </c>
       <c r="F158" s="5">
@@ -14960,7 +14960,7 @@
         <v/>
       </c>
       <c r="E159" s="5">
-        <f>IF(AND(C159="yes",ISNUMBER(G159)),MAX(DATE(2026,5,11),G159),"")</f>
+        <f>IF(AND(C159="yes",ISNUMBER(G159)),MAX(DATE(2026,5,13),G159),"")</f>
         <v/>
       </c>
       <c r="F159" s="5">
@@ -15051,7 +15051,7 @@
         <v/>
       </c>
       <c r="E160" s="5">
-        <f>IF(AND(C160="yes",ISNUMBER(G160)),MAX(DATE(2026,5,11),G160),"")</f>
+        <f>IF(AND(C160="yes",ISNUMBER(G160)),MAX(DATE(2026,5,13),G160),"")</f>
         <v/>
       </c>
       <c r="F160" s="5">
@@ -15142,7 +15142,7 @@
         <v/>
       </c>
       <c r="E161" s="5">
-        <f>IF(AND(C161="yes",ISNUMBER(G161)),MAX(DATE(2026,5,11),G161),"")</f>
+        <f>IF(AND(C161="yes",ISNUMBER(G161)),MAX(DATE(2026,5,13),G161),"")</f>
         <v/>
       </c>
       <c r="F161" s="5">
@@ -15233,7 +15233,7 @@
         <v/>
       </c>
       <c r="E162" s="5">
-        <f>IF(AND(C162="yes",ISNUMBER(G162)),MAX(DATE(2026,5,11),G162),"")</f>
+        <f>IF(AND(C162="yes",ISNUMBER(G162)),MAX(DATE(2026,5,13),G162),"")</f>
         <v/>
       </c>
       <c r="F162" s="5">
@@ -15324,7 +15324,7 @@
         <v/>
       </c>
       <c r="E163" s="5">
-        <f>IF(AND(C163="yes",ISNUMBER(G163)),MAX(DATE(2026,5,11),G163),"")</f>
+        <f>IF(AND(C163="yes",ISNUMBER(G163)),MAX(DATE(2026,5,13),G163),"")</f>
         <v/>
       </c>
       <c r="F163" s="5">
@@ -15415,7 +15415,7 @@
         <v/>
       </c>
       <c r="E164" s="5">
-        <f>IF(AND(C164="yes",ISNUMBER(G164)),MAX(DATE(2026,5,11),G164),"")</f>
+        <f>IF(AND(C164="yes",ISNUMBER(G164)),MAX(DATE(2026,5,13),G164),"")</f>
         <v/>
       </c>
       <c r="F164" s="5">
@@ -15506,7 +15506,7 @@
         <v/>
       </c>
       <c r="E165" s="5">
-        <f>IF(AND(C165="yes",ISNUMBER(G165)),MAX(DATE(2026,5,11),G165),"")</f>
+        <f>IF(AND(C165="yes",ISNUMBER(G165)),MAX(DATE(2026,5,13),G165),"")</f>
         <v/>
       </c>
       <c r="F165" s="5">
@@ -15597,7 +15597,7 @@
         <v/>
       </c>
       <c r="E166" s="5">
-        <f>IF(AND(C166="yes",ISNUMBER(G166)),MAX(DATE(2026,5,11),G166),"")</f>
+        <f>IF(AND(C166="yes",ISNUMBER(G166)),MAX(DATE(2026,5,13),G166),"")</f>
         <v/>
       </c>
       <c r="F166" s="5">
@@ -15688,7 +15688,7 @@
         <v/>
       </c>
       <c r="E167" s="5">
-        <f>IF(AND(C167="yes",ISNUMBER(G167)),MAX(DATE(2026,5,11),G167),"")</f>
+        <f>IF(AND(C167="yes",ISNUMBER(G167)),MAX(DATE(2026,5,13),G167),"")</f>
         <v/>
       </c>
       <c r="F167" s="5">
@@ -15779,7 +15779,7 @@
         <v/>
       </c>
       <c r="E168" s="5">
-        <f>IF(AND(C168="yes",ISNUMBER(G168)),MAX(DATE(2026,5,11),G168),"")</f>
+        <f>IF(AND(C168="yes",ISNUMBER(G168)),MAX(DATE(2026,5,13),G168),"")</f>
         <v/>
       </c>
       <c r="F168" s="5">
@@ -15870,7 +15870,7 @@
         <v/>
       </c>
       <c r="E169" s="5">
-        <f>IF(AND(C169="yes",ISNUMBER(G169)),MAX(DATE(2026,5,11),G169),"")</f>
+        <f>IF(AND(C169="yes",ISNUMBER(G169)),MAX(DATE(2026,5,13),G169),"")</f>
         <v/>
       </c>
       <c r="F169" s="5">
@@ -15961,7 +15961,7 @@
         <v/>
       </c>
       <c r="E170" s="5">
-        <f>IF(AND(C170="yes",ISNUMBER(G170)),MAX(DATE(2026,5,11),G170),"")</f>
+        <f>IF(AND(C170="yes",ISNUMBER(G170)),MAX(DATE(2026,5,13),G170),"")</f>
         <v/>
       </c>
       <c r="F170" s="5">
@@ -16052,7 +16052,7 @@
         <v/>
       </c>
       <c r="E171" s="5">
-        <f>IF(AND(C171="yes",ISNUMBER(G171)),MAX(DATE(2026,5,11),G171),"")</f>
+        <f>IF(AND(C171="yes",ISNUMBER(G171)),MAX(DATE(2026,5,13),G171),"")</f>
         <v/>
       </c>
       <c r="F171" s="5">
@@ -16143,7 +16143,7 @@
         <v/>
       </c>
       <c r="E172" s="5">
-        <f>IF(AND(C172="yes",ISNUMBER(G172)),MAX(DATE(2026,5,11),G172),"")</f>
+        <f>IF(AND(C172="yes",ISNUMBER(G172)),MAX(DATE(2026,5,13),G172),"")</f>
         <v/>
       </c>
       <c r="F172" s="5">
@@ -16234,7 +16234,7 @@
         <v/>
       </c>
       <c r="E173" s="5">
-        <f>IF(AND(C173="yes",ISNUMBER(G173)),MAX(DATE(2026,5,11),G173),"")</f>
+        <f>IF(AND(C173="yes",ISNUMBER(G173)),MAX(DATE(2026,5,13),G173),"")</f>
         <v/>
       </c>
       <c r="F173" s="5">
@@ -16325,7 +16325,7 @@
         <v/>
       </c>
       <c r="E174" s="5">
-        <f>IF(AND(C174="yes",ISNUMBER(G174)),MAX(DATE(2026,5,11),G174),"")</f>
+        <f>IF(AND(C174="yes",ISNUMBER(G174)),MAX(DATE(2026,5,13),G174),"")</f>
         <v/>
       </c>
       <c r="F174" s="5">
@@ -16416,7 +16416,7 @@
         <v/>
       </c>
       <c r="E175" s="5">
-        <f>IF(AND(C175="yes",ISNUMBER(G175)),MAX(DATE(2026,5,11),G175),"")</f>
+        <f>IF(AND(C175="yes",ISNUMBER(G175)),MAX(DATE(2026,5,13),G175),"")</f>
         <v/>
       </c>
       <c r="F175" s="5">
@@ -16507,7 +16507,7 @@
         <v/>
       </c>
       <c r="E176" s="5">
-        <f>IF(AND(C176="yes",ISNUMBER(G176)),MAX(DATE(2026,5,11),G176),"")</f>
+        <f>IF(AND(C176="yes",ISNUMBER(G176)),MAX(DATE(2026,5,13),G176),"")</f>
         <v/>
       </c>
       <c r="F176" s="5">
@@ -16598,7 +16598,7 @@
         <v/>
       </c>
       <c r="E177" s="5">
-        <f>IF(AND(C177="yes",ISNUMBER(G177)),MAX(DATE(2026,5,11),G177),"")</f>
+        <f>IF(AND(C177="yes",ISNUMBER(G177)),MAX(DATE(2026,5,13),G177),"")</f>
         <v/>
       </c>
       <c r="F177" s="5">
@@ -16689,7 +16689,7 @@
         <v/>
       </c>
       <c r="E178" s="5">
-        <f>IF(AND(C178="yes",ISNUMBER(G178)),MAX(DATE(2026,5,11),G178),"")</f>
+        <f>IF(AND(C178="yes",ISNUMBER(G178)),MAX(DATE(2026,5,13),G178),"")</f>
         <v/>
       </c>
       <c r="F178" s="5">
@@ -16780,7 +16780,7 @@
         <v/>
       </c>
       <c r="E179" s="5">
-        <f>IF(AND(C179="yes",ISNUMBER(G179)),MAX(DATE(2026,5,11),G179),"")</f>
+        <f>IF(AND(C179="yes",ISNUMBER(G179)),MAX(DATE(2026,5,13),G179),"")</f>
         <v/>
       </c>
       <c r="F179" s="5">
@@ -16871,7 +16871,7 @@
         <v/>
       </c>
       <c r="E180" s="5">
-        <f>IF(AND(C180="yes",ISNUMBER(G180)),MAX(DATE(2026,5,11),G180),"")</f>
+        <f>IF(AND(C180="yes",ISNUMBER(G180)),MAX(DATE(2026,5,13),G180),"")</f>
         <v/>
       </c>
       <c r="F180" s="5">
@@ -16962,7 +16962,7 @@
         <v/>
       </c>
       <c r="E181" s="5">
-        <f>IF(AND(C181="yes",ISNUMBER(G181)),MAX(DATE(2026,5,11),G181),"")</f>
+        <f>IF(AND(C181="yes",ISNUMBER(G181)),MAX(DATE(2026,5,13),G181),"")</f>
         <v/>
       </c>
       <c r="F181" s="5">
@@ -17053,7 +17053,7 @@
         <v/>
       </c>
       <c r="E182" s="5">
-        <f>IF(AND(C182="yes",ISNUMBER(G182)),MAX(DATE(2026,5,11),G182),"")</f>
+        <f>IF(AND(C182="yes",ISNUMBER(G182)),MAX(DATE(2026,5,13),G182),"")</f>
         <v/>
       </c>
       <c r="F182" s="5">
@@ -17144,7 +17144,7 @@
         <v/>
       </c>
       <c r="E183" s="5">
-        <f>IF(AND(C183="yes",ISNUMBER(G183)),MAX(DATE(2026,5,11),G183),"")</f>
+        <f>IF(AND(C183="yes",ISNUMBER(G183)),MAX(DATE(2026,5,13),G183),"")</f>
         <v/>
       </c>
       <c r="F183" s="5">
@@ -17235,7 +17235,7 @@
         <v/>
       </c>
       <c r="E184" s="5">
-        <f>IF(AND(C184="yes",ISNUMBER(G184)),MAX(DATE(2026,5,11),G184),"")</f>
+        <f>IF(AND(C184="yes",ISNUMBER(G184)),MAX(DATE(2026,5,13),G184),"")</f>
         <v/>
       </c>
       <c r="F184" s="5">
@@ -17326,7 +17326,7 @@
         <v/>
       </c>
       <c r="E185" s="5">
-        <f>IF(AND(C185="yes",ISNUMBER(G185)),MAX(DATE(2026,5,11),G185),"")</f>
+        <f>IF(AND(C185="yes",ISNUMBER(G185)),MAX(DATE(2026,5,13),G185),"")</f>
         <v/>
       </c>
       <c r="F185" s="5">
@@ -17417,7 +17417,7 @@
         <v/>
       </c>
       <c r="E186" s="5">
-        <f>IF(AND(C186="yes",ISNUMBER(G186)),MAX(DATE(2026,5,11),G186),"")</f>
+        <f>IF(AND(C186="yes",ISNUMBER(G186)),MAX(DATE(2026,5,13),G186),"")</f>
         <v/>
       </c>
       <c r="F186" s="5">
@@ -17508,7 +17508,7 @@
         <v/>
       </c>
       <c r="E187" s="5">
-        <f>IF(AND(C187="yes",ISNUMBER(G187)),MAX(DATE(2026,5,11),G187),"")</f>
+        <f>IF(AND(C187="yes",ISNUMBER(G187)),MAX(DATE(2026,5,13),G187),"")</f>
         <v/>
       </c>
       <c r="F187" s="5">
@@ -17599,7 +17599,7 @@
         <v/>
       </c>
       <c r="E188" s="5">
-        <f>IF(AND(C188="yes",ISNUMBER(G188)),MAX(DATE(2026,5,11),G188),"")</f>
+        <f>IF(AND(C188="yes",ISNUMBER(G188)),MAX(DATE(2026,5,13),G188),"")</f>
         <v/>
       </c>
       <c r="F188" s="5">
@@ -17690,7 +17690,7 @@
         <v/>
       </c>
       <c r="E189" s="5">
-        <f>IF(AND(C189="yes",ISNUMBER(G189)),MAX(DATE(2026,5,11),G189),"")</f>
+        <f>IF(AND(C189="yes",ISNUMBER(G189)),MAX(DATE(2026,5,13),G189),"")</f>
         <v/>
       </c>
       <c r="F189" s="5">
@@ -17781,7 +17781,7 @@
         <v/>
       </c>
       <c r="E190" s="5">
-        <f>IF(AND(C190="yes",ISNUMBER(G190)),MAX(DATE(2026,5,11),G190),"")</f>
+        <f>IF(AND(C190="yes",ISNUMBER(G190)),MAX(DATE(2026,5,13),G190),"")</f>
         <v/>
       </c>
       <c r="F190" s="5">
@@ -17872,7 +17872,7 @@
         <v/>
       </c>
       <c r="E191" s="5">
-        <f>IF(AND(C191="yes",ISNUMBER(G191)),MAX(DATE(2026,5,11),G191),"")</f>
+        <f>IF(AND(C191="yes",ISNUMBER(G191)),MAX(DATE(2026,5,13),G191),"")</f>
         <v/>
       </c>
       <c r="F191" s="5">
@@ -17963,7 +17963,7 @@
         <v/>
       </c>
       <c r="E192" s="5">
-        <f>IF(AND(C192="yes",ISNUMBER(G192)),MAX(DATE(2026,5,11),G192),"")</f>
+        <f>IF(AND(C192="yes",ISNUMBER(G192)),MAX(DATE(2026,5,13),G192),"")</f>
         <v/>
       </c>
       <c r="F192" s="5">
@@ -18054,7 +18054,7 @@
         <v/>
       </c>
       <c r="E193" s="5">
-        <f>IF(AND(C193="yes",ISNUMBER(G193)),MAX(DATE(2026,5,11),G193),"")</f>
+        <f>IF(AND(C193="yes",ISNUMBER(G193)),MAX(DATE(2026,5,13),G193),"")</f>
         <v/>
       </c>
       <c r="F193" s="5">
@@ -18145,7 +18145,7 @@
         <v/>
       </c>
       <c r="E194" s="5">
-        <f>IF(AND(C194="yes",ISNUMBER(G194)),MAX(DATE(2026,5,11),G194),"")</f>
+        <f>IF(AND(C194="yes",ISNUMBER(G194)),MAX(DATE(2026,5,13),G194),"")</f>
         <v/>
       </c>
       <c r="F194" s="5">
@@ -18236,7 +18236,7 @@
         <v/>
       </c>
       <c r="E195" s="5">
-        <f>IF(AND(C195="yes",ISNUMBER(G195)),MAX(DATE(2026,5,11),G195),"")</f>
+        <f>IF(AND(C195="yes",ISNUMBER(G195)),MAX(DATE(2026,5,13),G195),"")</f>
         <v/>
       </c>
       <c r="F195" s="5">
@@ -18327,7 +18327,7 @@
         <v/>
       </c>
       <c r="E196" s="5">
-        <f>IF(AND(C196="yes",ISNUMBER(G196)),MAX(DATE(2026,5,11),G196),"")</f>
+        <f>IF(AND(C196="yes",ISNUMBER(G196)),MAX(DATE(2026,5,13),G196),"")</f>
         <v/>
       </c>
       <c r="F196" s="5">
@@ -18418,7 +18418,7 @@
         <v/>
       </c>
       <c r="E197" s="5">
-        <f>IF(AND(C197="yes",ISNUMBER(G197)),MAX(DATE(2026,5,11),G197),"")</f>
+        <f>IF(AND(C197="yes",ISNUMBER(G197)),MAX(DATE(2026,5,13),G197),"")</f>
         <v/>
       </c>
       <c r="F197" s="5">
@@ -18509,7 +18509,7 @@
         <v/>
       </c>
       <c r="E198" s="5">
-        <f>IF(AND(C198="yes",ISNUMBER(G198)),MAX(DATE(2026,5,11),G198),"")</f>
+        <f>IF(AND(C198="yes",ISNUMBER(G198)),MAX(DATE(2026,5,13),G198),"")</f>
         <v/>
       </c>
       <c r="F198" s="5">
@@ -18600,7 +18600,7 @@
         <v/>
       </c>
       <c r="E199" s="5">
-        <f>IF(AND(C199="yes",ISNUMBER(G199)),MAX(DATE(2026,5,11),G199),"")</f>
+        <f>IF(AND(C199="yes",ISNUMBER(G199)),MAX(DATE(2026,5,13),G199),"")</f>
         <v/>
       </c>
       <c r="F199" s="5">
@@ -18691,7 +18691,7 @@
         <v/>
       </c>
       <c r="E200" s="5">
-        <f>IF(AND(C200="yes",ISNUMBER(G200)),MAX(DATE(2026,5,11),G200),"")</f>
+        <f>IF(AND(C200="yes",ISNUMBER(G200)),MAX(DATE(2026,5,13),G200),"")</f>
         <v/>
       </c>
       <c r="F200" s="5">
@@ -18782,7 +18782,7 @@
         <v/>
       </c>
       <c r="E201" s="5">
-        <f>IF(AND(C201="yes",ISNUMBER(G201)),MAX(DATE(2026,5,11),G201),"")</f>
+        <f>IF(AND(C201="yes",ISNUMBER(G201)),MAX(DATE(2026,5,13),G201),"")</f>
         <v/>
       </c>
       <c r="F201" s="5">
@@ -18873,7 +18873,7 @@
         <v/>
       </c>
       <c r="E202" s="5">
-        <f>IF(AND(C202="yes",ISNUMBER(G202)),MAX(DATE(2026,5,11),G202),"")</f>
+        <f>IF(AND(C202="yes",ISNUMBER(G202)),MAX(DATE(2026,5,13),G202),"")</f>
         <v/>
       </c>
       <c r="F202" s="5">
@@ -18964,7 +18964,7 @@
         <v/>
       </c>
       <c r="E203" s="5">
-        <f>IF(AND(C203="yes",ISNUMBER(G203)),MAX(DATE(2026,5,11),G203),"")</f>
+        <f>IF(AND(C203="yes",ISNUMBER(G203)),MAX(DATE(2026,5,13),G203),"")</f>
         <v/>
       </c>
       <c r="F203" s="5">
@@ -19055,7 +19055,7 @@
         <v/>
       </c>
       <c r="E204" s="5">
-        <f>IF(AND(C204="yes",ISNUMBER(G204)),MAX(DATE(2026,5,11),G204),"")</f>
+        <f>IF(AND(C204="yes",ISNUMBER(G204)),MAX(DATE(2026,5,13),G204),"")</f>
         <v/>
       </c>
       <c r="F204" s="5">
@@ -19146,7 +19146,7 @@
         <v/>
       </c>
       <c r="E205" s="5">
-        <f>IF(AND(C205="yes",ISNUMBER(G205)),MAX(DATE(2026,5,11),G205),"")</f>
+        <f>IF(AND(C205="yes",ISNUMBER(G205)),MAX(DATE(2026,5,13),G205),"")</f>
         <v/>
       </c>
       <c r="F205" s="5">
@@ -19237,7 +19237,7 @@
         <v/>
       </c>
       <c r="E206" s="5">
-        <f>IF(AND(C206="yes",ISNUMBER(G206)),MAX(DATE(2026,5,11),G206),"")</f>
+        <f>IF(AND(C206="yes",ISNUMBER(G206)),MAX(DATE(2026,5,13),G206),"")</f>
         <v/>
       </c>
       <c r="F206" s="5">
@@ -19328,7 +19328,7 @@
         <v/>
       </c>
       <c r="E207" s="5">
-        <f>IF(AND(C207="yes",ISNUMBER(G207)),MAX(DATE(2026,5,11),G207),"")</f>
+        <f>IF(AND(C207="yes",ISNUMBER(G207)),MAX(DATE(2026,5,13),G207),"")</f>
         <v/>
       </c>
       <c r="F207" s="5">
@@ -19419,7 +19419,7 @@
         <v/>
       </c>
       <c r="E208" s="5">
-        <f>IF(AND(C208="yes",ISNUMBER(G208)),MAX(DATE(2026,5,11),G208),"")</f>
+        <f>IF(AND(C208="yes",ISNUMBER(G208)),MAX(DATE(2026,5,13),G208),"")</f>
         <v/>
       </c>
       <c r="F208" s="5">
@@ -19510,7 +19510,7 @@
         <v/>
       </c>
       <c r="E209" s="5">
-        <f>IF(AND(C209="yes",ISNUMBER(G209)),MAX(DATE(2026,5,11),G209),"")</f>
+        <f>IF(AND(C209="yes",ISNUMBER(G209)),MAX(DATE(2026,5,13),G209),"")</f>
         <v/>
       </c>
       <c r="F209" s="5">
@@ -19601,7 +19601,7 @@
         <v/>
       </c>
       <c r="E210" s="5">
-        <f>IF(AND(C210="yes",ISNUMBER(G210)),MAX(DATE(2026,5,11),G210),"")</f>
+        <f>IF(AND(C210="yes",ISNUMBER(G210)),MAX(DATE(2026,5,13),G210),"")</f>
         <v/>
       </c>
       <c r="F210" s="5">
@@ -19692,7 +19692,7 @@
         <v/>
       </c>
       <c r="E211" s="5">
-        <f>IF(AND(C211="yes",ISNUMBER(G211)),MAX(DATE(2026,5,11),G211),"")</f>
+        <f>IF(AND(C211="yes",ISNUMBER(G211)),MAX(DATE(2026,5,13),G211),"")</f>
         <v/>
       </c>
       <c r="F211" s="5">
@@ -19783,7 +19783,7 @@
         <v/>
       </c>
       <c r="E212" s="5">
-        <f>IF(AND(C212="yes",ISNUMBER(G212)),MAX(DATE(2026,5,11),G212),"")</f>
+        <f>IF(AND(C212="yes",ISNUMBER(G212)),MAX(DATE(2026,5,13),G212),"")</f>
         <v/>
       </c>
       <c r="F212" s="5">
@@ -19874,7 +19874,7 @@
         <v/>
       </c>
       <c r="E213" s="5">
-        <f>IF(AND(C213="yes",ISNUMBER(G213)),MAX(DATE(2026,5,11),G213),"")</f>
+        <f>IF(AND(C213="yes",ISNUMBER(G213)),MAX(DATE(2026,5,13),G213),"")</f>
         <v/>
       </c>
       <c r="F213" s="5">
@@ -19965,7 +19965,7 @@
         <v/>
       </c>
       <c r="E214" s="5">
-        <f>IF(AND(C214="yes",ISNUMBER(G214)),MAX(DATE(2026,5,11),G214),"")</f>
+        <f>IF(AND(C214="yes",ISNUMBER(G214)),MAX(DATE(2026,5,13),G214),"")</f>
         <v/>
       </c>
       <c r="F214" s="5">
@@ -20056,7 +20056,7 @@
         <v/>
       </c>
       <c r="E215" s="5">
-        <f>IF(AND(C215="yes",ISNUMBER(G215)),MAX(DATE(2026,5,11),G215),"")</f>
+        <f>IF(AND(C215="yes",ISNUMBER(G215)),MAX(DATE(2026,5,13),G215),"")</f>
         <v/>
       </c>
       <c r="F215" s="5">
@@ -20147,7 +20147,7 @@
         <v/>
       </c>
       <c r="E216" s="5">
-        <f>IF(AND(C216="yes",ISNUMBER(G216)),MAX(DATE(2026,5,11),G216),"")</f>
+        <f>IF(AND(C216="yes",ISNUMBER(G216)),MAX(DATE(2026,5,13),G216),"")</f>
         <v/>
       </c>
       <c r="F216" s="5">
@@ -20238,7 +20238,7 @@
         <v/>
       </c>
       <c r="E217" s="5">
-        <f>IF(AND(C217="yes",ISNUMBER(G217)),MAX(DATE(2026,5,11),G217),"")</f>
+        <f>IF(AND(C217="yes",ISNUMBER(G217)),MAX(DATE(2026,5,13),G217),"")</f>
         <v/>
       </c>
       <c r="F217" s="5">
@@ -20329,7 +20329,7 @@
         <v/>
       </c>
       <c r="E218" s="5">
-        <f>IF(AND(C218="yes",ISNUMBER(G218)),MAX(DATE(2026,5,11),G218),"")</f>
+        <f>IF(AND(C218="yes",ISNUMBER(G218)),MAX(DATE(2026,5,13),G218),"")</f>
         <v/>
       </c>
       <c r="F218" s="5">
@@ -20420,7 +20420,7 @@
         <v/>
       </c>
       <c r="E219" s="5">
-        <f>IF(AND(C219="yes",ISNUMBER(G219)),MAX(DATE(2026,5,11),G219),"")</f>
+        <f>IF(AND(C219="yes",ISNUMBER(G219)),MAX(DATE(2026,5,13),G219),"")</f>
         <v/>
       </c>
       <c r="F219" s="5">
@@ -20511,7 +20511,7 @@
         <v/>
       </c>
       <c r="E220" s="5">
-        <f>IF(AND(C220="yes",ISNUMBER(G220)),MAX(DATE(2026,5,11),G220),"")</f>
+        <f>IF(AND(C220="yes",ISNUMBER(G220)),MAX(DATE(2026,5,13),G220),"")</f>
         <v/>
       </c>
       <c r="F220" s="5">
@@ -20602,7 +20602,7 @@
         <v/>
       </c>
       <c r="E221" s="5">
-        <f>IF(AND(C221="yes",ISNUMBER(G221)),MAX(DATE(2026,5,11),G221),"")</f>
+        <f>IF(AND(C221="yes",ISNUMBER(G221)),MAX(DATE(2026,5,13),G221),"")</f>
         <v/>
       </c>
       <c r="F221" s="5">
@@ -20693,7 +20693,7 @@
         <v/>
       </c>
       <c r="E222" s="5">
-        <f>IF(AND(C222="yes",ISNUMBER(G222)),MAX(DATE(2026,5,11),G222),"")</f>
+        <f>IF(AND(C222="yes",ISNUMBER(G222)),MAX(DATE(2026,5,13),G222),"")</f>
         <v/>
       </c>
       <c r="F222" s="5">
@@ -20784,7 +20784,7 @@
         <v/>
       </c>
       <c r="E223" s="5">
-        <f>IF(AND(C223="yes",ISNUMBER(G223)),MAX(DATE(2026,5,11),G223),"")</f>
+        <f>IF(AND(C223="yes",ISNUMBER(G223)),MAX(DATE(2026,5,13),G223),"")</f>
         <v/>
       </c>
       <c r="F223" s="5">
@@ -20875,7 +20875,7 @@
         <v/>
       </c>
       <c r="E224" s="5">
-        <f>IF(AND(C224="yes",ISNUMBER(G224)),MAX(DATE(2026,5,11),G224),"")</f>
+        <f>IF(AND(C224="yes",ISNUMBER(G224)),MAX(DATE(2026,5,13),G224),"")</f>
         <v/>
       </c>
       <c r="F224" s="5">
@@ -20966,7 +20966,7 @@
         <v/>
       </c>
       <c r="E225" s="5">
-        <f>IF(AND(C225="yes",ISNUMBER(G225)),MAX(DATE(2026,5,11),G225),"")</f>
+        <f>IF(AND(C225="yes",ISNUMBER(G225)),MAX(DATE(2026,5,13),G225),"")</f>
         <v/>
       </c>
       <c r="F225" s="5">
@@ -21057,7 +21057,7 @@
         <v/>
       </c>
       <c r="E226" s="5">
-        <f>IF(AND(C226="yes",ISNUMBER(G226)),MAX(DATE(2026,5,11),G226),"")</f>
+        <f>IF(AND(C226="yes",ISNUMBER(G226)),MAX(DATE(2026,5,13),G226),"")</f>
         <v/>
       </c>
       <c r="F226" s="5">
@@ -21148,7 +21148,7 @@
         <v/>
       </c>
       <c r="E227" s="5">
-        <f>IF(AND(C227="yes",ISNUMBER(G227)),MAX(DATE(2026,5,11),G227),"")</f>
+        <f>IF(AND(C227="yes",ISNUMBER(G227)),MAX(DATE(2026,5,13),G227),"")</f>
         <v/>
       </c>
       <c r="F227" s="5">
@@ -21239,7 +21239,7 @@
         <v/>
       </c>
       <c r="E228" s="5">
-        <f>IF(AND(C228="yes",ISNUMBER(G228)),MAX(DATE(2026,5,11),G228),"")</f>
+        <f>IF(AND(C228="yes",ISNUMBER(G228)),MAX(DATE(2026,5,13),G228),"")</f>
         <v/>
       </c>
       <c r="F228" s="5">
@@ -21330,7 +21330,7 @@
         <v/>
       </c>
       <c r="E229" s="5">
-        <f>IF(AND(C229="yes",ISNUMBER(G229)),MAX(DATE(2026,5,11),G229),"")</f>
+        <f>IF(AND(C229="yes",ISNUMBER(G229)),MAX(DATE(2026,5,13),G229),"")</f>
         <v/>
       </c>
       <c r="F229" s="5">
@@ -21421,7 +21421,7 @@
         <v/>
       </c>
       <c r="E230" s="5">
-        <f>IF(AND(C230="yes",ISNUMBER(G230)),MAX(DATE(2026,5,11),G230),"")</f>
+        <f>IF(AND(C230="yes",ISNUMBER(G230)),MAX(DATE(2026,5,13),G230),"")</f>
         <v/>
       </c>
       <c r="F230" s="5">
@@ -21512,7 +21512,7 @@
         <v/>
       </c>
       <c r="E231" s="5">
-        <f>IF(AND(C231="yes",ISNUMBER(G231)),MAX(DATE(2026,5,11),G231),"")</f>
+        <f>IF(AND(C231="yes",ISNUMBER(G231)),MAX(DATE(2026,5,13),G231),"")</f>
         <v/>
       </c>
       <c r="F231" s="5">
@@ -21603,7 +21603,7 @@
         <v/>
       </c>
       <c r="E232" s="5">
-        <f>IF(AND(C232="yes",ISNUMBER(G232)),MAX(DATE(2026,5,11),G232),"")</f>
+        <f>IF(AND(C232="yes",ISNUMBER(G232)),MAX(DATE(2026,5,13),G232),"")</f>
         <v/>
       </c>
       <c r="F232" s="5">
@@ -21690,7 +21690,7 @@
         <v/>
       </c>
       <c r="E233" s="5">
-        <f>IF(AND(C233="yes",ISNUMBER(G233)),MAX(DATE(2026,5,11),G233),"")</f>
+        <f>IF(AND(C233="yes",ISNUMBER(G233)),MAX(DATE(2026,5,13),G233),"")</f>
         <v/>
       </c>
       <c r="F233" s="5">
@@ -21777,7 +21777,7 @@
         <v/>
       </c>
       <c r="E234" s="5">
-        <f>IF(AND(C234="yes",ISNUMBER(G234)),MAX(DATE(2026,5,11),G234),"")</f>
+        <f>IF(AND(C234="yes",ISNUMBER(G234)),MAX(DATE(2026,5,13),G234),"")</f>
         <v/>
       </c>
       <c r="F234" s="5">
@@ -21868,7 +21868,7 @@
         <v/>
       </c>
       <c r="E235" s="5">
-        <f>IF(AND(C235="yes",ISNUMBER(G235)),MAX(DATE(2026,5,11),G235),"")</f>
+        <f>IF(AND(C235="yes",ISNUMBER(G235)),MAX(DATE(2026,5,13),G235),"")</f>
         <v/>
       </c>
       <c r="F235" s="5">
@@ -21959,7 +21959,7 @@
         <v/>
       </c>
       <c r="E236" s="5">
-        <f>IF(AND(C236="yes",ISNUMBER(G236)),MAX(DATE(2026,5,11),G236),"")</f>
+        <f>IF(AND(C236="yes",ISNUMBER(G236)),MAX(DATE(2026,5,13),G236),"")</f>
         <v/>
       </c>
       <c r="F236" s="5">
@@ -22050,7 +22050,7 @@
         <v/>
       </c>
       <c r="E237" s="5">
-        <f>IF(AND(C237="yes",ISNUMBER(G237)),MAX(DATE(2026,5,11),G237),"")</f>
+        <f>IF(AND(C237="yes",ISNUMBER(G237)),MAX(DATE(2026,5,13),G237),"")</f>
         <v/>
       </c>
       <c r="F237" s="5">
@@ -22141,7 +22141,7 @@
         <v/>
       </c>
       <c r="E238" s="5">
-        <f>IF(AND(C238="yes",ISNUMBER(G238)),MAX(DATE(2026,5,11),G238),"")</f>
+        <f>IF(AND(C238="yes",ISNUMBER(G238)),MAX(DATE(2026,5,13),G238),"")</f>
         <v/>
       </c>
       <c r="F238" s="5">
@@ -22232,7 +22232,7 @@
         <v/>
       </c>
       <c r="E239" s="5">
-        <f>IF(AND(C239="yes",ISNUMBER(G239)),MAX(DATE(2026,5,11),G239),"")</f>
+        <f>IF(AND(C239="yes",ISNUMBER(G239)),MAX(DATE(2026,5,13),G239),"")</f>
         <v/>
       </c>
       <c r="F239" s="5">
@@ -22323,7 +22323,7 @@
         <v/>
       </c>
       <c r="E240" s="5">
-        <f>IF(AND(C240="yes",ISNUMBER(G240)),MAX(DATE(2026,5,11),G240),"")</f>
+        <f>IF(AND(C240="yes",ISNUMBER(G240)),MAX(DATE(2026,5,13),G240),"")</f>
         <v/>
       </c>
       <c r="F240" s="5">
@@ -22414,7 +22414,7 @@
         <v/>
       </c>
       <c r="E241" s="5">
-        <f>IF(AND(C241="yes",ISNUMBER(G241)),MAX(DATE(2026,5,11),G241),"")</f>
+        <f>IF(AND(C241="yes",ISNUMBER(G241)),MAX(DATE(2026,5,13),G241),"")</f>
         <v/>
       </c>
       <c r="F241" s="5">
@@ -22505,7 +22505,7 @@
         <v/>
       </c>
       <c r="E242" s="5">
-        <f>IF(AND(C242="yes",ISNUMBER(G242)),MAX(DATE(2026,5,11),G242),"")</f>
+        <f>IF(AND(C242="yes",ISNUMBER(G242)),MAX(DATE(2026,5,13),G242),"")</f>
         <v/>
       </c>
       <c r="F242" s="5">
@@ -22596,7 +22596,7 @@
         <v/>
       </c>
       <c r="E243" s="5">
-        <f>IF(AND(C243="yes",ISNUMBER(G243)),MAX(DATE(2026,5,11),G243),"")</f>
+        <f>IF(AND(C243="yes",ISNUMBER(G243)),MAX(DATE(2026,5,13),G243),"")</f>
         <v/>
       </c>
       <c r="F243" s="5">
@@ -22687,7 +22687,7 @@
         <v/>
       </c>
       <c r="E244" s="5">
-        <f>IF(AND(C244="yes",ISNUMBER(G244)),MAX(DATE(2026,5,11),G244),"")</f>
+        <f>IF(AND(C244="yes",ISNUMBER(G244)),MAX(DATE(2026,5,13),G244),"")</f>
         <v/>
       </c>
       <c r="F244" s="5">
@@ -22778,7 +22778,7 @@
         <v/>
       </c>
       <c r="E245" s="5">
-        <f>IF(AND(C245="yes",ISNUMBER(G245)),MAX(DATE(2026,5,11),G245),"")</f>
+        <f>IF(AND(C245="yes",ISNUMBER(G245)),MAX(DATE(2026,5,13),G245),"")</f>
         <v/>
       </c>
       <c r="F245" s="5">
@@ -22869,7 +22869,7 @@
         <v/>
       </c>
       <c r="E246" s="5">
-        <f>IF(AND(C246="yes",ISNUMBER(G246)),MAX(DATE(2026,5,11),G246),"")</f>
+        <f>IF(AND(C246="yes",ISNUMBER(G246)),MAX(DATE(2026,5,13),G246),"")</f>
         <v/>
       </c>
       <c r="F246" s="5">
@@ -22960,7 +22960,7 @@
         <v/>
       </c>
       <c r="E247" s="5">
-        <f>IF(AND(C247="yes",ISNUMBER(G247)),MAX(DATE(2026,5,11),G247),"")</f>
+        <f>IF(AND(C247="yes",ISNUMBER(G247)),MAX(DATE(2026,5,13),G247),"")</f>
         <v/>
       </c>
       <c r="F247" s="5">
@@ -23051,7 +23051,7 @@
         <v/>
       </c>
       <c r="E248" s="5">
-        <f>IF(AND(C248="yes",ISNUMBER(G248)),MAX(DATE(2026,5,11),G248),"")</f>
+        <f>IF(AND(C248="yes",ISNUMBER(G248)),MAX(DATE(2026,5,13),G248),"")</f>
         <v/>
       </c>
       <c r="F248" s="5">
@@ -23142,7 +23142,7 @@
         <v/>
       </c>
       <c r="E249" s="5">
-        <f>IF(AND(C249="yes",ISNUMBER(G249)),MAX(DATE(2026,5,11),G249),"")</f>
+        <f>IF(AND(C249="yes",ISNUMBER(G249)),MAX(DATE(2026,5,13),G249),"")</f>
         <v/>
       </c>
       <c r="F249" s="5">
@@ -23233,7 +23233,7 @@
         <v/>
       </c>
       <c r="E250" s="5">
-        <f>IF(AND(C250="yes",ISNUMBER(G250)),MAX(DATE(2026,5,11),G250),"")</f>
+        <f>IF(AND(C250="yes",ISNUMBER(G250)),MAX(DATE(2026,5,13),G250),"")</f>
         <v/>
       </c>
       <c r="F250" s="5">
@@ -23256,7 +23256,7 @@
       </c>
       <c r="J250" s="2" t="inlineStr">
         <is>
-          <t>N/A — no P batch assigned</t>
+          <t>P060212</t>
         </is>
       </c>
       <c r="K250" s="2" t="inlineStr">
@@ -23324,7 +23324,7 @@
         <v/>
       </c>
       <c r="E251" s="5">
-        <f>IF(AND(C251="yes",ISNUMBER(G251)),MAX(DATE(2026,5,11),G251),"")</f>
+        <f>IF(AND(C251="yes",ISNUMBER(G251)),MAX(DATE(2026,5,13),G251),"")</f>
         <v/>
       </c>
       <c r="F251" s="5">
@@ -23347,7 +23347,7 @@
       </c>
       <c r="J251" s="2" t="inlineStr">
         <is>
-          <t>N/A — no P batch assigned</t>
+          <t>P060212</t>
         </is>
       </c>
       <c r="K251" s="2" t="inlineStr">
@@ -23415,7 +23415,7 @@
         <v/>
       </c>
       <c r="E252" s="5">
-        <f>IF(AND(C252="yes",ISNUMBER(G252)),MAX(DATE(2026,5,11),G252),"")</f>
+        <f>IF(AND(C252="yes",ISNUMBER(G252)),MAX(DATE(2026,5,13),G252),"")</f>
         <v/>
       </c>
       <c r="F252" s="5">
@@ -23506,7 +23506,7 @@
         <v/>
       </c>
       <c r="E253" s="5">
-        <f>IF(AND(C253="yes",ISNUMBER(G253)),MAX(DATE(2026,5,11),G253),"")</f>
+        <f>IF(AND(C253="yes",ISNUMBER(G253)),MAX(DATE(2026,5,13),G253),"")</f>
         <v/>
       </c>
       <c r="F253" s="5">
@@ -23597,7 +23597,7 @@
         <v/>
       </c>
       <c r="E254" s="5">
-        <f>IF(AND(C254="yes",ISNUMBER(G254)),MAX(DATE(2026,5,11),G254),"")</f>
+        <f>IF(AND(C254="yes",ISNUMBER(G254)),MAX(DATE(2026,5,13),G254),"")</f>
         <v/>
       </c>
       <c r="F254" s="5">
@@ -23688,7 +23688,7 @@
         <v/>
       </c>
       <c r="E255" s="5">
-        <f>IF(AND(C255="yes",ISNUMBER(G255)),MAX(DATE(2026,5,11),G255),"")</f>
+        <f>IF(AND(C255="yes",ISNUMBER(G255)),MAX(DATE(2026,5,13),G255),"")</f>
         <v/>
       </c>
       <c r="F255" s="5">
@@ -23779,7 +23779,7 @@
         <v/>
       </c>
       <c r="E256" s="5">
-        <f>IF(AND(C256="yes",ISNUMBER(G256)),MAX(DATE(2026,5,11),G256),"")</f>
+        <f>IF(AND(C256="yes",ISNUMBER(G256)),MAX(DATE(2026,5,13),G256),"")</f>
         <v/>
       </c>
       <c r="F256" s="5">
@@ -23870,7 +23870,7 @@
         <v/>
       </c>
       <c r="E257" s="5">
-        <f>IF(AND(C257="yes",ISNUMBER(G257)),MAX(DATE(2026,5,11),G257),"")</f>
+        <f>IF(AND(C257="yes",ISNUMBER(G257)),MAX(DATE(2026,5,13),G257),"")</f>
         <v/>
       </c>
       <c r="F257" s="5">
@@ -23961,7 +23961,7 @@
         <v/>
       </c>
       <c r="E258" s="5">
-        <f>IF(AND(C258="yes",ISNUMBER(G258)),MAX(DATE(2026,5,11),G258),"")</f>
+        <f>IF(AND(C258="yes",ISNUMBER(G258)),MAX(DATE(2026,5,13),G258),"")</f>
         <v/>
       </c>
       <c r="F258" s="5">
@@ -24052,7 +24052,7 @@
         <v/>
       </c>
       <c r="E259" s="5">
-        <f>IF(AND(C259="yes",ISNUMBER(G259)),MAX(DATE(2026,5,11),G259),"")</f>
+        <f>IF(AND(C259="yes",ISNUMBER(G259)),MAX(DATE(2026,5,13),G259),"")</f>
         <v/>
       </c>
       <c r="F259" s="5">
@@ -24143,7 +24143,7 @@
         <v/>
       </c>
       <c r="E260" s="5">
-        <f>IF(AND(C260="yes",ISNUMBER(G260)),MAX(DATE(2026,5,11),G260),"")</f>
+        <f>IF(AND(C260="yes",ISNUMBER(G260)),MAX(DATE(2026,5,13),G260),"")</f>
         <v/>
       </c>
       <c r="F260" s="5">
@@ -24234,7 +24234,7 @@
         <v/>
       </c>
       <c r="E261" s="5">
-        <f>IF(AND(C261="yes",ISNUMBER(G261)),MAX(DATE(2026,5,11),G261),"")</f>
+        <f>IF(AND(C261="yes",ISNUMBER(G261)),MAX(DATE(2026,5,13),G261),"")</f>
         <v/>
       </c>
       <c r="F261" s="5">
@@ -24325,7 +24325,7 @@
         <v/>
       </c>
       <c r="E262" s="5">
-        <f>IF(AND(C262="yes",ISNUMBER(G262)),MAX(DATE(2026,5,11),G262),"")</f>
+        <f>IF(AND(C262="yes",ISNUMBER(G262)),MAX(DATE(2026,5,13),G262),"")</f>
         <v/>
       </c>
       <c r="F262" s="5">
@@ -24416,7 +24416,7 @@
         <v/>
       </c>
       <c r="E263" s="5">
-        <f>IF(AND(C263="yes",ISNUMBER(G263)),MAX(DATE(2026,5,11),G263),"")</f>
+        <f>IF(AND(C263="yes",ISNUMBER(G263)),MAX(DATE(2026,5,13),G263),"")</f>
         <v/>
       </c>
       <c r="F263" s="5">
@@ -24507,7 +24507,7 @@
         <v/>
       </c>
       <c r="E264" s="5">
-        <f>IF(AND(C264="yes",ISNUMBER(G264)),MAX(DATE(2026,5,11),G264),"")</f>
+        <f>IF(AND(C264="yes",ISNUMBER(G264)),MAX(DATE(2026,5,13),G264),"")</f>
         <v/>
       </c>
       <c r="F264" s="5">
@@ -24598,7 +24598,7 @@
         <v/>
       </c>
       <c r="E265" s="5">
-        <f>IF(AND(C265="yes",ISNUMBER(G265)),MAX(DATE(2026,5,11),G265),"")</f>
+        <f>IF(AND(C265="yes",ISNUMBER(G265)),MAX(DATE(2026,5,13),G265),"")</f>
         <v/>
       </c>
       <c r="F265" s="5">
@@ -24689,7 +24689,7 @@
         <v/>
       </c>
       <c r="E266" s="5">
-        <f>IF(AND(C266="yes",ISNUMBER(G266)),MAX(DATE(2026,5,11),G266),"")</f>
+        <f>IF(AND(C266="yes",ISNUMBER(G266)),MAX(DATE(2026,5,13),G266),"")</f>
         <v/>
       </c>
       <c r="F266" s="5">
@@ -24780,7 +24780,7 @@
         <v/>
       </c>
       <c r="E267" s="5">
-        <f>IF(AND(C267="yes",ISNUMBER(G267)),MAX(DATE(2026,5,11),G267),"")</f>
+        <f>IF(AND(C267="yes",ISNUMBER(G267)),MAX(DATE(2026,5,13),G267),"")</f>
         <v/>
       </c>
       <c r="F267" s="5">
@@ -24871,7 +24871,7 @@
         <v/>
       </c>
       <c r="E268" s="5">
-        <f>IF(AND(C268="yes",ISNUMBER(G268)),MAX(DATE(2026,5,11),G268),"")</f>
+        <f>IF(AND(C268="yes",ISNUMBER(G268)),MAX(DATE(2026,5,13),G268),"")</f>
         <v/>
       </c>
       <c r="F268" s="5">
@@ -24962,7 +24962,7 @@
         <v/>
       </c>
       <c r="E269" s="5">
-        <f>IF(AND(C269="yes",ISNUMBER(G269)),MAX(DATE(2026,5,11),G269),"")</f>
+        <f>IF(AND(C269="yes",ISNUMBER(G269)),MAX(DATE(2026,5,13),G269),"")</f>
         <v/>
       </c>
       <c r="F269" s="5">
@@ -25053,7 +25053,7 @@
         <v/>
       </c>
       <c r="E270" s="5">
-        <f>IF(AND(C270="yes",ISNUMBER(G270)),MAX(DATE(2026,5,11),G270),"")</f>
+        <f>IF(AND(C270="yes",ISNUMBER(G270)),MAX(DATE(2026,5,13),G270),"")</f>
         <v/>
       </c>
       <c r="F270" s="5">
@@ -25144,7 +25144,7 @@
         <v/>
       </c>
       <c r="E271" s="5">
-        <f>IF(AND(C271="yes",ISNUMBER(G271)),MAX(DATE(2026,5,11),G271),"")</f>
+        <f>IF(AND(C271="yes",ISNUMBER(G271)),MAX(DATE(2026,5,13),G271),"")</f>
         <v/>
       </c>
       <c r="F271" s="5">
@@ -25235,7 +25235,7 @@
         <v/>
       </c>
       <c r="E272" s="5">
-        <f>IF(AND(C272="yes",ISNUMBER(G272)),MAX(DATE(2026,5,11),G272),"")</f>
+        <f>IF(AND(C272="yes",ISNUMBER(G272)),MAX(DATE(2026,5,13),G272),"")</f>
         <v/>
       </c>
       <c r="F272" s="5">
@@ -25322,7 +25322,7 @@
         <v/>
       </c>
       <c r="E273" s="5">
-        <f>IF(AND(C273="yes",ISNUMBER(G273)),MAX(DATE(2026,5,11),G273),"")</f>
+        <f>IF(AND(C273="yes",ISNUMBER(G273)),MAX(DATE(2026,5,13),G273),"")</f>
         <v/>
       </c>
       <c r="F273" s="5">
@@ -25409,7 +25409,7 @@
         <v/>
       </c>
       <c r="E274" s="5">
-        <f>IF(AND(C274="yes",ISNUMBER(G274)),MAX(DATE(2026,5,11),G274),"")</f>
+        <f>IF(AND(C274="yes",ISNUMBER(G274)),MAX(DATE(2026,5,13),G274),"")</f>
         <v/>
       </c>
       <c r="F274" s="5">
@@ -25496,7 +25496,7 @@
         <v/>
       </c>
       <c r="E275" s="5">
-        <f>IF(AND(C275="yes",ISNUMBER(G275)),MAX(DATE(2026,5,11),G275),"")</f>
+        <f>IF(AND(C275="yes",ISNUMBER(G275)),MAX(DATE(2026,5,13),G275),"")</f>
         <v/>
       </c>
       <c r="F275" s="5">
@@ -25583,7 +25583,7 @@
         <v/>
       </c>
       <c r="E276" s="5">
-        <f>IF(AND(C276="yes",ISNUMBER(G276)),MAX(DATE(2026,5,11),G276),"")</f>
+        <f>IF(AND(C276="yes",ISNUMBER(G276)),MAX(DATE(2026,5,13),G276),"")</f>
         <v/>
       </c>
       <c r="F276" s="5">
@@ -25670,7 +25670,7 @@
         <v/>
       </c>
       <c r="E277" s="5">
-        <f>IF(AND(C277="yes",ISNUMBER(G277)),MAX(DATE(2026,5,11),G277),"")</f>
+        <f>IF(AND(C277="yes",ISNUMBER(G277)),MAX(DATE(2026,5,13),G277),"")</f>
         <v/>
       </c>
       <c r="F277" s="5">
@@ -25757,7 +25757,7 @@
         <v/>
       </c>
       <c r="E278" s="5">
-        <f>IF(AND(C278="yes",ISNUMBER(G278)),MAX(DATE(2026,5,11),G278),"")</f>
+        <f>IF(AND(C278="yes",ISNUMBER(G278)),MAX(DATE(2026,5,13),G278),"")</f>
         <v/>
       </c>
       <c r="F278" s="5">
@@ -25848,7 +25848,7 @@
         <v/>
       </c>
       <c r="E279" s="5">
-        <f>IF(AND(C279="yes",ISNUMBER(G279)),MAX(DATE(2026,5,11),G279),"")</f>
+        <f>IF(AND(C279="yes",ISNUMBER(G279)),MAX(DATE(2026,5,13),G279),"")</f>
         <v/>
       </c>
       <c r="F279" s="5">
@@ -25939,7 +25939,7 @@
         <v/>
       </c>
       <c r="E280" s="5">
-        <f>IF(AND(C280="yes",ISNUMBER(G280)),MAX(DATE(2026,5,11),G280),"")</f>
+        <f>IF(AND(C280="yes",ISNUMBER(G280)),MAX(DATE(2026,5,13),G280),"")</f>
         <v/>
       </c>
       <c r="F280" s="5">
@@ -26030,7 +26030,7 @@
         <v/>
       </c>
       <c r="E281" s="5">
-        <f>IF(AND(C281="yes",ISNUMBER(G281)),MAX(DATE(2026,5,11),G281),"")</f>
+        <f>IF(AND(C281="yes",ISNUMBER(G281)),MAX(DATE(2026,5,13),G281),"")</f>
         <v/>
       </c>
       <c r="F281" s="5">
@@ -26121,7 +26121,7 @@
         <v/>
       </c>
       <c r="E282" s="5">
-        <f>IF(AND(C282="yes",ISNUMBER(G282)),MAX(DATE(2026,5,11),G282),"")</f>
+        <f>IF(AND(C282="yes",ISNUMBER(G282)),MAX(DATE(2026,5,13),G282),"")</f>
         <v/>
       </c>
       <c r="F282" s="5">
@@ -26212,7 +26212,7 @@
         <v/>
       </c>
       <c r="E283" s="5">
-        <f>IF(AND(C283="yes",ISNUMBER(G283)),MAX(DATE(2026,5,11),G283),"")</f>
+        <f>IF(AND(C283="yes",ISNUMBER(G283)),MAX(DATE(2026,5,13),G283),"")</f>
         <v/>
       </c>
       <c r="F283" s="5">
@@ -26303,7 +26303,7 @@
         <v/>
       </c>
       <c r="E284" s="5">
-        <f>IF(AND(C284="yes",ISNUMBER(G284)),MAX(DATE(2026,5,11),G284),"")</f>
+        <f>IF(AND(C284="yes",ISNUMBER(G284)),MAX(DATE(2026,5,13),G284),"")</f>
         <v/>
       </c>
       <c r="F284" s="5">
@@ -26394,7 +26394,7 @@
         <v/>
       </c>
       <c r="E285" s="5">
-        <f>IF(AND(C285="yes",ISNUMBER(G285)),MAX(DATE(2026,5,11),G285),"")</f>
+        <f>IF(AND(C285="yes",ISNUMBER(G285)),MAX(DATE(2026,5,13),G285),"")</f>
         <v/>
       </c>
       <c r="F285" s="5">
@@ -26485,7 +26485,7 @@
         <v/>
       </c>
       <c r="E286" s="5">
-        <f>IF(AND(C286="yes",ISNUMBER(G286)),MAX(DATE(2026,5,11),G286),"")</f>
+        <f>IF(AND(C286="yes",ISNUMBER(G286)),MAX(DATE(2026,5,13),G286),"")</f>
         <v/>
       </c>
       <c r="F286" s="5">
@@ -26576,7 +26576,7 @@
         <v/>
       </c>
       <c r="E287" s="5">
-        <f>IF(AND(C287="yes",ISNUMBER(G287)),MAX(DATE(2026,5,11),G287),"")</f>
+        <f>IF(AND(C287="yes",ISNUMBER(G287)),MAX(DATE(2026,5,13),G287),"")</f>
         <v/>
       </c>
       <c r="F287" s="5">
@@ -26667,7 +26667,7 @@
         <v/>
       </c>
       <c r="E288" s="5">
-        <f>IF(AND(C288="yes",ISNUMBER(G288)),MAX(DATE(2026,5,11),G288),"")</f>
+        <f>IF(AND(C288="yes",ISNUMBER(G288)),MAX(DATE(2026,5,13),G288),"")</f>
         <v/>
       </c>
       <c r="F288" s="5">
@@ -26758,7 +26758,7 @@
         <v/>
       </c>
       <c r="E289" s="5">
-        <f>IF(AND(C289="yes",ISNUMBER(G289)),MAX(DATE(2026,5,11),G289),"")</f>
+        <f>IF(AND(C289="yes",ISNUMBER(G289)),MAX(DATE(2026,5,13),G289),"")</f>
         <v/>
       </c>
       <c r="F289" s="5">
@@ -26833,7 +26833,7 @@
     <row r="291" ht="96" customHeight="1">
       <c r="A291" s="9" t="inlineStr">
         <is>
-          <t>Head of QC, 05.09.2026: preliminary iCoA issuance register. Document codes iCoA-PP_26-nnn (nnn = 001 … 999), one series for the year of issue, assigned in the order the certificates can be issued: by the earliest permissible issue date, then by the basis date (the first day of packaging, when the sample is taken). Every printed issue date lies in [11.05.2026 … the day of signing] — the CoQ SOP came into use on 11.05.2026 and no document is post-dated — so the preliminary date is the SOP floor, or the last day of packaging where that is later; QC sets the real date at issue (documents may be issued in batches: one date, sequential numbers). No number is reserved for a row that cannot be issued yet: a lot without a packaging date, a held result, and every retest iCoA (identification A, B and foreign matter are tested at the retest sampling, whose date is not on the desk). Where a CNP certificate reports all three, no iCoA is needed. The plan's references of 31.08.2026 (iCoA-PP-YYYY-NNNN) are superseded by these codes and kept beside them. Identification C is not on the iCoA: the CoQ cites the cannabinoid-assay eCoA named here. TWO CERTIFICATES PER P LOT (05.09.2026): identification A and B on the P01-02 master, foreign matter on the P07 master. FORMULAS: No. counts the issuable rows above it, the code is built from No., the earliest and preliminary dates from the SOP floor and the packaging dates looked up on Batch Dates by P batch (or CU batch); insert a row, set Issuable to yes, and every code beneath moves by one — the iCoA Issuance sheet and the tracker cite the register by KEY, so they follow. Rows are not re-sorted by a formula: a changed date is a manual move.</t>
+          <t>Head of QC, 05.09.2026: preliminary iCoA issuance register. Document codes iCoA-PP_26-nnn (nnn = 001 … 999), one series for the year of issue, assigned in the order the certificates can be issued: by the earliest permissible issue date, then by the basis date (the first day of packaging, when the sample is taken). Every printed issue date lies in [11.05.2026 … the day of signing] — the CoQ SOP came into use on 11.05.2026 and no document is post-dated — and, Head of QC 05.09.2026, every certificate whose lot was packed before the SOP floor is issued on ONE day, 13.05.2026 (a Wednesday), in chronological order of packaging; the lots packed after it follow, each on its last day of packaging, the numbers running on. No number is reserved for a row that cannot be issued yet: a lot without a packaging date, a held result, and every retest iCoA (identification A, B and foreign matter are tested at the retest sampling, whose date is not on the desk). Where a CNP certificate reports all three, no iCoA is needed. The plan's references of 31.08.2026 (iCoA-PP-YYYY-NNNN) are superseded by these codes and kept beside them. Identification C is not on the iCoA: the CoQ cites the cannabinoid-assay eCoA named here. TWO CERTIFICATES PER P LOT (05.09.2026): identification A and B on the P01-02 master, foreign matter on the P07 master. FORMULAS: No. counts the issuable rows above it, the code is built from No., the earliest and preliminary dates from the SOP floor and the packaging dates looked up on Batch Dates by P batch (or CU batch); insert a row, set Issuable to yes, and every code beneath moves by one — the iCoA Issuance sheet and the tracker cite the register by KEY, so they follow. Rows are not re-sorted by a formula: a changed date is a manual move.</t>
         </is>
       </c>
     </row>
@@ -30211,7 +30211,7 @@
     <row r="2" ht="120" customHeight="1">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Head of QC, 05.09.2026: preliminary iCoA issuance register. Document codes iCoA-PP_26-nnn (nnn = 001 … 999), one series for the year of issue, assigned in the order the certificates can be issued: by the earliest permissible issue date, then by the basis date (the first day of packaging, when the sample is taken). Every printed issue date lies in [11.05.2026 … the day of signing] — the CoQ SOP came into use on 11.05.2026 and no document is post-dated — so the preliminary date is the SOP floor, or the last day of packaging where that is later; QC sets the real date at issue (documents may be issued in batches: one date, sequential numbers). No number is reserved for a row that cannot be issued yet: a lot without a packaging date, a held result, and every retest iCoA (identification A, B and foreign matter are tested at the retest sampling, whose date is not on the desk). Where a CNP certificate reports all three, no iCoA is needed. The plan's references of 31.08.2026 (iCoA-PP-YYYY-NNNN) are superseded by these codes and kept beside them. Identification C is not on the iCoA: the CoQ cites the cannabinoid-assay eCoA named here. TWO CERTIFICATES PER P LOT (05.09.2026): identification A and B on the P01-02 master, foreign matter on the P07 master. FORMULAS: No. counts the issuable rows above it, the code is built from No., the earliest and preliminary dates from the SOP floor and the packaging dates looked up on Batch Dates by P batch (or CU batch); insert a row, set Issuable to yes, and every code beneath moves by one — the iCoA Issuance sheet and the tracker cite the register by KEY, so they follow. Rows are not re-sorted by a formula: a changed date is a manual move.</t>
+          <t>Head of QC, 05.09.2026: preliminary iCoA issuance register. Document codes iCoA-PP_26-nnn (nnn = 001 … 999), one series for the year of issue, assigned in the order the certificates can be issued: by the earliest permissible issue date, then by the basis date (the first day of packaging, when the sample is taken). Every printed issue date lies in [11.05.2026 … the day of signing] — the CoQ SOP came into use on 11.05.2026 and no document is post-dated — and, Head of QC 05.09.2026, every certificate whose lot was packed before the SOP floor is issued on ONE day, 13.05.2026 (a Wednesday), in chronological order of packaging; the lots packed after it follow, each on its last day of packaging, the numbers running on. No number is reserved for a row that cannot be issued yet: a lot without a packaging date, a held result, and every retest iCoA (identification A, B and foreign matter are tested at the retest sampling, whose date is not on the desk). Where a CNP certificate reports all three, no iCoA is needed. The plan's references of 31.08.2026 (iCoA-PP-YYYY-NNNN) are superseded by these codes and kept beside them. Identification C is not on the iCoA: the CoQ cites the cannabinoid-assay eCoA named here. TWO CERTIFICATES PER P LOT (05.09.2026): identification A and B on the P01-02 master, foreign matter on the P07 master. FORMULAS: No. counts the issuable rows above it, the code is built from No., the earliest and preliminary dates from the SOP floor and the packaging dates looked up on Batch Dates by P batch (or CU batch); insert a row, set Issuable to yes, and every code beneath moves by one — the iCoA Issuance sheet and the tracker cite the register by KEY, so they follow. Rows are not re-sorted by a formula: a changed date is a manual move.</t>
         </is>
       </c>
     </row>

</xml_diff>